<commit_message>
girlievault: keyword research workbook rebuilt from the updated plan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -867,7 +867,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Women's Tracksuit Pants: How to Choose Your Fit</t>
+          <t>Workout Pants for Women: Fit That Moves With You</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>tracksuit pants for ladies</t>
+          <t>workout pants for women</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1255,10 +1255,10 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>3600</v>
+        <v>2900</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Workout Pants for Women: Fit That Moves With You</t>
+          <t>Best Butt-Lifting Leggings for a Sculpted, Confident Shape</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>workout pants for women</t>
+          <t>best butt lifting leggings</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -1301,10 +1301,10 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>2900</v>
+        <v>2400</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
@@ -1323,22 +1323,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Best Butt-Lifting Leggings for a Sculpted, Confident Shape</t>
+          <t>Workout Sets: The Girlie Vault Guide to Matched Activewear</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>best butt lifting leggings</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Leggings &amp; Bottoms</t>
+          <t>workout sets</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Matching Sets &amp; Outfits</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1347,14 +1347,14 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>2400</v>
+        <v>40500</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>40</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Workout Sets: The Girlie Vault Guide to Matched Activewear</t>
+          <t>What to Know Before Buying a Two-Piece Set</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>workout sets</t>
+          <t>two piece sets</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1393,10 +1393,10 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>40500</v>
+        <v>27100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>What to Know Before Buying a Two-Piece Set</t>
+          <t>White Two-Piece Sets: Styling a Fresh Coordinated Look</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>two piece sets</t>
+          <t>white two piece set</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -1430,23 +1430,23 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>27100</v>
+        <v>8100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>22</v>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>White Two-Piece Sets: Styling a Fresh Coordinated Look</t>
+          <t>Plus-Size Workout Clothes for Confident Movement</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>white two piece set</t>
+          <t>plus size workout clothes</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1485,14 +1485,14 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>45</v>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -1507,12 +1507,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Plus-Size Workout Clothes for Confident Movement</t>
+          <t>Matching Sets for Women Who Love Effortless Style</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>plus size workout clothes</t>
+          <t>sets for women</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -1531,14 +1531,14 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>40</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Matching Sets for Women Who Love Effortless Style</t>
+          <t>Women's Gym Dresses: How to Find Your Perfect Fit</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>sets for women</t>
+          <t>gym dress for ladies</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1577,14 +1577,14 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>5400</v>
+        <v>4400</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>47</v>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1599,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Women's Gym Dresses: How to Find Your Perfect Fit</t>
+          <t>Women's Jogger Sets: How to Pick One You Will Live In</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>gym dress for ladies</t>
+          <t>female jogger set</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -1619,18 +1619,18 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>28</v>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -1691,22 +1691,22 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>How to Style Yoga Flare Pants for Any Occasion</t>
+          <t>Cropped Tank Tops: How to Find Your Perfect Fit</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>yoga flare pants outfits</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>Matching Sets &amp; Outfits</t>
+          <t>cropped tank top</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Sports Bras &amp; Tops</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1715,14 +1715,14 @@
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>2400</v>
+        <v>4400</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>12</v>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Cropped Tank Tops: How to Find Your Perfect Fit</t>
+          <t>High-Support Sports Bras: Lock-In Coverage for Any Impact</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>cropped tank top</t>
+          <t>high sports bra support</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -1764,11 +1764,11 @@
         <v>4400</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="J26" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>37</v>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>High-Support Sports Bras: Lock-In Coverage for Any Impact</t>
+          <t>Plus-Size Sports Bras That Deliver Real Support</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>high sports bra support</t>
+          <t>plus size sports bra</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -1798,23 +1798,23 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
         <v>4400</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>27</v>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Plus-Size Sports Bras That Deliver Real Support</t>
+          <t>Yellow Tank Tops: Styling a Bright, Bold Basic</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>plus size sports bra</t>
+          <t>yellow tank top</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1853,10 +1853,10 @@
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
@@ -1875,12 +1875,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Yellow Tank Tops: Styling a Bright, Bold Basic</t>
+          <t>Cotton Sports Bras: Soft Support for Low-Impact Days</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>yellow tank top</t>
+          <t>cotton sports bra</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -1899,10 +1899,10 @@
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>3600</v>
+        <v>2900</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
@@ -1921,12 +1921,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Cotton Sports Bras: Soft Support for Low-Impact Days</t>
+          <t>Gym Hoodies: Choosing One for Warm-Ups and Cool-Downs</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>cotton sports bra</t>
+          <t>gym hoodies</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1948,7 +1948,7 @@
         <v>2900</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
@@ -1967,22 +1967,22 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>The Best Seamless Sports Bras for Everyday Comfort</t>
+          <t>What to Know Before You Buy a String Bikini</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>seamless sports bra</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Sports Bras &amp; Tops</t>
+          <t>string bikini</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Swimwear &amp; Beach</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1991,14 +1991,14 @@
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>1300</v>
+        <v>22200</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="J31" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>24</v>
+      </c>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -2013,12 +2013,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Tankini Swimsuits: How to Find Your Perfect Fit</t>
+          <t>High-Waisted Bikinis: Flattering Coverage With Confidence</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>tankini swimsuit</t>
+          <t>high waisted bikini</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2037,10 +2037,10 @@
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>22200</v>
+        <v>18100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>What to Know Before You Buy a String Bikini</t>
+          <t>The Best Tummy-Control Swimsuits for Every Body</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>string bikini</t>
+          <t>tummy control swimsuit</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -2074,19 +2074,19 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>22200</v>
+        <v>14800</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Bikinis: Flattering Coverage With Confidence</t>
+          <t>Black One-Piece Swimsuits: The Everyday Flattering Staple</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>high waisted bikini</t>
+          <t>black one piece swimsuit</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -2120,19 +2120,19 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>18100</v>
+        <v>8100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
@@ -2151,12 +2151,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>The Best Tummy-Control Swimsuits for Every Body</t>
+          <t>Bikini Bottoms: How to Find Your Most Flattering Cut</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>tummy control swimsuit</t>
+          <t>bikini bottoms</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2175,10 +2175,10 @@
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>14800</v>
+        <v>6600</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
@@ -2197,12 +2197,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Swim Shorts for Women: Comfort Meets Coverage</t>
+          <t>High-Waisted vs Mid-Rise Bikini Bottoms: Which Flatters You</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>swim shorts for women</t>
+          <t>high waisted bikini bottoms</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -2217,14 +2217,14 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>12100</v>
+        <v>6600</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
@@ -2243,12 +2243,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Swim Skirts: Flattering Coverage for Beach and Pool</t>
+          <t>Long-Sleeve Swimsuits: Coverage, Sun Protection, and Fit</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>swim skirt</t>
+          <t>long sleeve swimsuit</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -2258,23 +2258,23 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>9</v>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2289,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Black One-Piece Swimsuits: The Everyday Flattering Staple</t>
+          <t>Two-Piece Swimsuits: A Buyer's Guide for Women</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>black one piece swimsuit</t>
+          <t>two piece swimming costumes for ladies</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
@@ -2309,14 +2309,14 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>8100</v>
+        <v>5400</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
@@ -2335,12 +2335,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Bikini Bottoms: How to Find Your Most Flattering Cut</t>
+          <t>Long Torso Swimsuits: How to Find One That Actually Fits</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>bikini bottoms</t>
+          <t>long torso swimsuits</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -2355,18 +2355,18 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>6600</v>
+        <v>4400</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="J39" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>7</v>
+      </c>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2381,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted vs Mid-Rise Bikini Bottoms: Which Flatters You</t>
+          <t>Spring Break Swimwear: What to Pack and How to Choose</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>high waisted bikini bottoms</t>
+          <t>spring break swimwear</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -2396,23 +2396,23 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>6600</v>
+        <v>4400</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J40" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>9</v>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2427,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Two-Piece Swimsuits: A Buyer's Guide for Women</t>
+          <t>Full-Coverage Swimsuits: Comfort In and Out of the Water</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>two piece swimming costumes for ladies</t>
+          <t>full coverage swimsuit</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -2442,19 +2442,19 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>5400</v>
+        <v>3600</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H46" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H51" s="2" t="n">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H52" s="2" t="n">
@@ -2995,12 +2995,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>The Girlie Vault Guide to Flare Leggings</t>
+          <t>Athletic Shorts: Choosing the Right Pair for Every Workout</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>flare leggings</t>
+          <t>athletic shorts</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -3015,18 +3015,18 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>27100</v>
+        <v>22200</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="J53" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>48</v>
+      </c>
+      <c r="J53" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3041,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Athletic Shorts: Choosing the Right Pair for Every Workout</t>
+          <t>Straight-Leg Sweatpants: A Buyer's Guide to Fit and Fabric</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>athletic shorts</t>
+          <t>straight leg sweatpants</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -3061,18 +3061,18 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>22200</v>
+        <v>12100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="J54" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>15</v>
+      </c>
+      <c r="J54" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3087,12 +3087,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Straight-Leg Sweatpants: A Buyer's Guide to Fit and Fabric</t>
+          <t>The Best Compression Leggings for Squat-Proof Coverage</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>straight leg sweatpants</t>
+          <t>compression leggings</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
         <v>12100</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
@@ -3133,12 +3133,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>The Best Compression Leggings for Squat-Proof Coverage</t>
+          <t>Workout Shorts: Finding the Right Length and Fit</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>compression leggings</t>
+          <t>workout shorts</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3157,14 +3157,14 @@
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>12100</v>
+        <v>9900</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="J56" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>33</v>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Workout Shorts: Finding the Right Length and Fit</t>
+          <t>Leggings With Pockets: How to Find the Most Functional Pair</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>workout shorts</t>
+          <t>leggings with pockets</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -3199,14 +3199,14 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H57" s="2" t="n">
         <v>9900</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
@@ -3225,12 +3225,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Leggings With Pockets: How to Find the Most Functional Pair</t>
+          <t>Yoga Shorts: How to Pick Your Perfect Pair</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>leggings with pockets</t>
+          <t>yoga shorts</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
@@ -3249,14 +3249,14 @@
         </is>
       </c>
       <c r="H58" s="2" t="n">
-        <v>9900</v>
+        <v>6600</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>22</v>
+      </c>
+      <c r="J58" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Yoga Shorts: How to Pick Your Perfect Pair</t>
+          <t>High-Waisted Leggings for All-Day Comfort and Support</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>yoga shorts</t>
+          <t>high waisted leggings</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -3286,23 +3286,23 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H59" s="2" t="n">
         <v>6600</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="J59" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>35</v>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3317,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Leggings for All-Day Comfort and Support</t>
+          <t>Fold-Over Leggings: Choosing Your Comfiest Waistband</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>high waisted leggings</t>
+          <t>fold over leggings</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -3332,23 +3332,23 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>19</v>
+      </c>
+      <c r="J60" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Fold-Over Leggings: Choosing Your Comfiest Waistband</t>
+          <t>Women's Board Shorts: Active Coverage for Sun and Surf</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>fold over leggings</t>
+          <t>womens board shorts</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -3390,7 +3390,7 @@
         <v>5400</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
@@ -3409,12 +3409,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Women's Board Shorts: Active Coverage for Sun and Surf</t>
+          <t>Tummy-Control Leggings for Smooth, All-Day Support</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>womens board shorts</t>
+          <t>tummy control leggings</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3433,10 +3433,10 @@
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>5400</v>
+        <v>2900</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Tummy-Control Leggings for Smooth, All-Day Support</t>
+          <t>Legging Shorts: The Length Between Bike Shorts and Leggings</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>tummy control leggings</t>
+          <t>legging shorts</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
         <v>2900</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H69" s="2" t="n">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H70" s="2" t="n">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H75" s="2" t="n">
@@ -4053,12 +4053,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Cropped Pants for Women: Style Meets Movement</t>
+          <t>Plus-Size Graphic Tees: Fit, Print, and Everyday Wear</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>cropped pants for women</t>
+          <t>plus size graphic tees</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -4068,19 +4068,19 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H76" s="2" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J76" s="8" t="inlineStr">
         <is>
@@ -4099,12 +4099,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Best Sports Bras for Running: What to Look For</t>
+          <t>Cropped Pants for Women: Style Meets Movement</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>best sports bra for running</t>
+          <t>cropped pants for women</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
@@ -4126,7 +4126,7 @@
         <v>1900</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J77" s="8" t="inlineStr">
         <is>
@@ -4145,22 +4145,22 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Tankini Beachwear: Coverage and Confidence in One</t>
+          <t>Best Sports Bras for Running: What to Look For</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>tankini beachwear</t>
-        </is>
-      </c>
-      <c r="E78" s="13" t="inlineStr">
-        <is>
-          <t>Swimwear &amp; Beach</t>
+          <t>best sports bra for running</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>Sports Bras &amp; Tops</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4169,10 +4169,10 @@
         </is>
       </c>
       <c r="H78" s="2" t="n">
-        <v>6600</v>
+        <v>1900</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H79" s="2" t="n">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H81" s="2" t="n">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H82" s="2" t="n">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H83" s="2" t="n">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H84" s="2" t="n">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H85" s="2" t="n">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H87" s="2" t="n">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H88" s="2" t="n">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H89" s="2" t="n">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Branded</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -5009,7 +5009,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H96" s="2" t="n">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H99" s="2" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H100" s="2" t="n">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H102" s="2" t="n">
@@ -5311,12 +5311,12 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Seamless Leggings for a Smooth, Sculpted Fit</t>
+          <t>Leopard Print Leggings: How to Wear a Bold Pattern</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>seamless leggings</t>
+          <t>leopard print leggings</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
@@ -5335,14 +5335,14 @@
         </is>
       </c>
       <c r="H103" s="2" t="n">
-        <v>4400</v>
+        <v>1900</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="J103" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>24</v>
+      </c>
+      <c r="J103" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H106" s="2" t="n">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H107" s="2" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H109" s="2" t="n">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Transactional</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="H114" s="2" t="n">
@@ -6418,9 +6418,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -6670,9 +6670,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7146,9 +7146,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7958,9 +7958,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F63" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8994,9 +8994,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F100" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9442,9 +9442,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -11262,9 +11262,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F181" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -11542,9 +11542,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F191" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -13502,9 +13502,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F261" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -13558,9 +13558,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F263" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F263" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -14034,9 +14034,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F280" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F280" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -15322,9 +15322,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F326" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F326" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -15546,9 +15546,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F334" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F334" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -21729,8 +21729,8 @@
     <row r="14" ht="65" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>BoFu (53) — category buying guides for shoppers ready to purchase.
-MoFu (48) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
+          <t>BoFu (52) — category buying guides for shoppers ready to purchase.
+MoFu (49) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
 ToFu (19) — education and styling that builds topical authority and earns citations.
 The MoFu/ToFu weighting is deliberate: those terms are winnable at a young domain and are exactly what AI engines cite when shoppers ask for recommendations.</t>
         </is>

</xml_diff>

<commit_message>
girlievault: keyword workbook rebuilt, no refreshes in the plan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -1323,12 +1323,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Workout Sets: The Girlie Vault Guide to Matched Activewear</t>
+          <t>What to Know Before Buying a Two-Piece Set</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>workout sets</t>
+          <t>two piece sets</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1347,10 +1347,10 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>40500</v>
+        <v>27100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>What to Know Before Buying a Two-Piece Set</t>
+          <t>White Two-Piece Sets: Styling a Fresh Coordinated Look</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>two piece sets</t>
+          <t>white two piece set</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1393,14 +1393,14 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>27100</v>
+        <v>8100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>22</v>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>White Two-Piece Sets: Styling a Fresh Coordinated Look</t>
+          <t>Plus-Size Activewear That Moves: A Fit and Fabric Guide</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>white two piece set</t>
+          <t>plus size workout clothes</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1439,14 +1439,14 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>45</v>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Plus-Size Workout Clothes for Confident Movement</t>
+          <t>Matching Sets for Women Who Love Effortless Style</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>plus size workout clothes</t>
+          <t>sets for women</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1485,14 +1485,14 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>40</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -1507,12 +1507,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Matching Sets for Women Who Love Effortless Style</t>
+          <t>Women's Gym Dresses: How to Find Your Perfect Fit</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>sets for women</t>
+          <t>gym dress for ladies</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1531,14 +1531,14 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>5400</v>
+        <v>4400</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>47</v>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Women's Gym Dresses: How to Find Your Perfect Fit</t>
+          <t>Women's Jogger Sets: How to Pick One You Will Live In</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>gym dress for ladies</t>
+          <t>female jogger set</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -1577,14 +1577,14 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>28</v>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1599,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Women's Jogger Sets: How to Pick One You Will Live In</t>
+          <t>Building a Workout Routine You Can Stick To</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>female jogger set</t>
+          <t>workout routine for women</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1623,14 +1623,14 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>3600</v>
+        <v>2900</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>46</v>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Building a Workout Routine You Can Stick To</t>
+          <t>Cropped Tank Tops: How to Find Your Perfect Fit</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>workout routine for women</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>Matching Sets &amp; Outfits</t>
+          <t>cropped tank top</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Sports Bras &amp; Tops</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1669,14 +1669,14 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>2900</v>
+        <v>4400</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="J24" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>12</v>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Cropped Tank Tops: How to Find Your Perfect Fit</t>
+          <t>High-Support Sports Bras: Lock-In Coverage for Any Impact</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>cropped tank top</t>
+          <t>high sports bra support</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -1718,11 +1718,11 @@
         <v>4400</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="J25" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>37</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>High-Support Sports Bras: Lock-In Coverage for Any Impact</t>
+          <t>Plus-Size Sports Bras That Deliver Real Support</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>high sports bra support</t>
+          <t>plus size sports bra</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1764,11 +1764,11 @@
         <v>4400</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>27</v>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Plus-Size Sports Bras That Deliver Real Support</t>
+          <t>Yellow Tank Tops: Styling a Bright, Bold Basic</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>plus size sports bra</t>
+          <t>yellow tank top</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1807,10 +1807,10 @@
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Yellow Tank Tops: Styling a Bright, Bold Basic</t>
+          <t>Cotton Sports Bras: Soft Support for Low-Impact Days</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>yellow tank top</t>
+          <t>cotton sports bra</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -1853,10 +1853,10 @@
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>3600</v>
+        <v>2900</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
@@ -1875,12 +1875,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Cotton Sports Bras: Soft Support for Low-Impact Days</t>
+          <t>Gym Hoodies: Choosing One for Warm-Ups and Cool-Downs</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>cotton sports bra</t>
+          <t>gym hoodies</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1902,7 +1902,7 @@
         <v>2900</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
@@ -1921,22 +1921,22 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Gym Hoodies: Choosing One for Warm-Ups and Cool-Downs</t>
+          <t>What to Know Before You Buy a String Bikini</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>gym hoodies</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>Sports Bras &amp; Tops</t>
+          <t>string bikini</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Swimwear &amp; Beach</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1945,10 +1945,10 @@
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>2900</v>
+        <v>22200</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
@@ -1967,12 +1967,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>What to Know Before You Buy a String Bikini</t>
+          <t>High-Waisted Bikinis: Flattering Coverage With Confidence</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>string bikini</t>
+          <t>high waisted bikini</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1991,10 +1991,10 @@
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>22200</v>
+        <v>18100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
@@ -2013,12 +2013,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Bikinis: Flattering Coverage With Confidence</t>
+          <t>The Best Tummy-Control Swimsuits for Every Body</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>high waisted bikini</t>
+          <t>tummy control swimsuit</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -2037,10 +2037,10 @@
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>18100</v>
+        <v>14800</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>The Best Tummy-Control Swimsuits for Every Body</t>
+          <t>Black One-Piece Swimsuits: The Everyday Flattering Staple</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>tummy control swimsuit</t>
+          <t>black one piece swimsuit</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2083,10 +2083,10 @@
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>14800</v>
+        <v>8100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Black One-Piece Swimsuits: The Everyday Flattering Staple</t>
+          <t>Bikini Bottoms: How to Find Your Most Flattering Cut</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>black one piece swimsuit</t>
+          <t>bikini bottoms</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -2129,10 +2129,10 @@
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
@@ -2151,12 +2151,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Bikini Bottoms: How to Find Your Most Flattering Cut</t>
+          <t>High-Waisted vs Mid-Rise Bikini Bottoms: Which Flatters You</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>bikini bottoms</t>
+          <t>high waisted bikini bottoms</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2178,7 +2178,7 @@
         <v>6600</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
@@ -2197,12 +2197,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted vs Mid-Rise Bikini Bottoms: Which Flatters You</t>
+          <t>Long-Sleeve Swimsuits: Coverage, Sun Protection, and Fit</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>high waisted bikini bottoms</t>
+          <t>long sleeve swimsuit</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -2224,11 +2224,11 @@
         <v>6600</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J36" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>9</v>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -2243,12 +2243,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Long-Sleeve Swimsuits: Coverage, Sun Protection, and Fit</t>
+          <t>Two-Piece Swimsuits: A Buyer's Guide for Women</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>long sleeve swimsuit</t>
+          <t>two piece swimming costumes for ladies</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2267,14 +2267,14 @@
         </is>
       </c>
       <c r="H37" s="2" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="J37" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>27</v>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2289,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Two-Piece Swimsuits: A Buyer's Guide for Women</t>
+          <t>Long Torso Swimsuits: How to Find One That Actually Fits</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>two piece swimming costumes for ladies</t>
+          <t>long torso swimsuits</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
@@ -2313,14 +2313,14 @@
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>5400</v>
+        <v>4400</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="J38" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>7</v>
+      </c>
+      <c r="J38" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -2335,12 +2335,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Long Torso Swimsuits: How to Find One That Actually Fits</t>
+          <t>Spring Break Swimwear: What to Pack and How to Choose</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>long torso swimsuits</t>
+          <t>spring break swimwear</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2362,7 +2362,7 @@
         <v>4400</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J39" s="12" t="inlineStr">
         <is>
@@ -2381,12 +2381,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Spring Break Swimwear: What to Pack and How to Choose</t>
+          <t>Full-Coverage Swimsuits: Comfort In and Out of the Water</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>spring break swimwear</t>
+          <t>full coverage swimsuit</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2405,14 +2405,14 @@
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="J40" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>16</v>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -2427,12 +2427,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Full-Coverage Swimsuits: Comfort In and Out of the Water</t>
+          <t>Bikini Tops for a Smaller Bust: How to Find Your Fit</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>full coverage swimsuit</t>
+          <t>bikinis to suit small bust</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2451,10 +2451,10 @@
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>3600</v>
+        <v>2900</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Leggings for All-Day Comfort and Support</t>
+          <t>Fold-Over Leggings: Choosing Your Comfiest Waistband</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>high waisted leggings</t>
+          <t>fold over leggings</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -3295,14 +3295,14 @@
         </is>
       </c>
       <c r="H59" s="2" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="J59" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>19</v>
+      </c>
+      <c r="J59" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3317,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Fold-Over Leggings: Choosing Your Comfiest Waistband</t>
+          <t>Tummy-Control Leggings for Smooth, All-Day Support</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>fold over leggings</t>
+          <t>tummy control leggings</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3341,10 +3341,10 @@
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>5400</v>
+        <v>2900</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
@@ -3363,12 +3363,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Women's Board Shorts: Active Coverage for Sun and Surf</t>
+          <t>Legging Shorts: The Length Between Bike Shorts and Leggings</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>womens board shorts</t>
+          <t>legging shorts</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -3387,10 +3387,10 @@
         </is>
       </c>
       <c r="H61" s="2" t="n">
-        <v>5400</v>
+        <v>2900</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
@@ -3409,22 +3409,22 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Tummy-Control Leggings for Smooth, All-Day Support</t>
+          <t>Matching Sets for Women: Finding Your Perfect Pairing</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>tummy control leggings</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="inlineStr">
-        <is>
-          <t>Leggings &amp; Bottoms</t>
+          <t>matching sets women</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Matching Sets &amp; Outfits</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3433,14 +3433,14 @@
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>2900</v>
+        <v>14800</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="J62" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>38</v>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -3455,22 +3455,22 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Legging Shorts: The Length Between Bike Shorts and Leggings</t>
+          <t>How to Put Together Pilates Outfits You Feel Good In</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>legging shorts</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>Leggings &amp; Bottoms</t>
+          <t>pilates outfits</t>
+        </is>
+      </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>Matching Sets &amp; Outfits</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="H63" s="2" t="n">
-        <v>2900</v>
+        <v>6600</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
@@ -3501,12 +3501,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Matching Sets for Women: Finding Your Perfect Pairing</t>
+          <t>Summer Sets: Easy Coordinated Warm-Weather Outfits</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>matching sets women</t>
+          <t>summer sets</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
@@ -3525,14 +3525,14 @@
         </is>
       </c>
       <c r="H64" s="2" t="n">
-        <v>14800</v>
+        <v>5400</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="J64" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>28</v>
+      </c>
+      <c r="J64" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3547,12 +3547,12 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>How to Put Together Pilates Outfits You Feel Good In</t>
+          <t>Yoga Clothes for Women Who Value Comfort and Stretch</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>pilates outfits</t>
+          <t>yoga clothes for women</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -3571,14 +3571,14 @@
         </is>
       </c>
       <c r="H65" s="2" t="n">
-        <v>6600</v>
+        <v>4400</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="J65" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>32</v>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -3593,12 +3593,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Summer Sets: Easy Coordinated Warm-Weather Outfits</t>
+          <t>Going-Out Sets: Matching Pieces That Work Past the Gym</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>summer sets</t>
+          <t>going out sets</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -3617,10 +3617,10 @@
         </is>
       </c>
       <c r="H66" s="2" t="n">
-        <v>5400</v>
+        <v>3600</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="J66" s="8" t="inlineStr">
         <is>
@@ -3639,12 +3639,12 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Yoga Clothes for Women Who Value Comfort and Stretch</t>
+          <t>Women's Gym Sets: Pieces That Work as Hard as You</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>yoga clothes for women</t>
+          <t>gym sets for women</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
@@ -3663,10 +3663,10 @@
         </is>
       </c>
       <c r="H67" s="2" t="n">
-        <v>4400</v>
+        <v>2900</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
@@ -3685,12 +3685,12 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Women's Gym Sets: Pieces That Work as Hard as You</t>
+          <t>How to Build a Workout Plan Women Can Stick To</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>gym sets for women</t>
+          <t>workout plan for ladies</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -3709,14 +3709,14 @@
         </is>
       </c>
       <c r="H68" s="2" t="n">
-        <v>2900</v>
+        <v>2400</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="J68" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>26</v>
+      </c>
+      <c r="J68" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3731,22 +3731,22 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>How to Build a Workout Plan Women Can Stick To</t>
+          <t>Racerback Bras: How to Choose the Right Support</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>workout plan for ladies</t>
-        </is>
-      </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>Matching Sets &amp; Outfits</t>
+          <t>racerback bra</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>Sports Bras &amp; Tops</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -3755,10 +3755,10 @@
         </is>
       </c>
       <c r="H69" s="2" t="n">
-        <v>2400</v>
+        <v>8100</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="J69" s="8" t="inlineStr">
         <is>
@@ -3777,12 +3777,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Racerback Bras: How to Choose the Right Support</t>
+          <t>Tank Tops With Built-In Bras: Finding Your Perfect Fit</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>racerback bra</t>
+          <t>tank top with built in bra</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -3801,10 +3801,10 @@
         </is>
       </c>
       <c r="H70" s="2" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="J70" s="8" t="inlineStr">
         <is>
@@ -3823,12 +3823,12 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Tank Tops With Built-In Bras: Finding Your Perfect Fit</t>
+          <t>Racerback Tanks: Finding Your Best Fit and Feel</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>tank top with built in bra</t>
+          <t>racerback tank</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -3847,10 +3847,10 @@
         </is>
       </c>
       <c r="H71" s="2" t="n">
-        <v>6600</v>
+        <v>4400</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J71" s="8" t="inlineStr">
         <is>
@@ -3869,12 +3869,12 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Racerback Tanks: Finding Your Best Fit and Feel</t>
+          <t>Push-Up Sports Bras: How to Find Support and Shape</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>racerback tank</t>
+          <t>push up sports bra</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -3893,10 +3893,10 @@
         </is>
       </c>
       <c r="H72" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="J72" s="8" t="inlineStr">
         <is>
@@ -3915,12 +3915,12 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Push-Up Sports Bras: How to Find Support and Shape</t>
+          <t>The Best Compression Sports Bras for High-Impact Support</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>push up sports bra</t>
+          <t>compression sports bra</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -3939,10 +3939,10 @@
         </is>
       </c>
       <c r="H73" s="2" t="n">
-        <v>3600</v>
+        <v>2900</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="J73" s="8" t="inlineStr">
         <is>
@@ -3961,12 +3961,12 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>The Best Compression Sports Bras for High-Impact Support</t>
+          <t>Cute Hooded Sweatshirts for Women to Layer and Lounge</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>compression sports bra</t>
+          <t>cute hooded sweatshirts for women</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -3985,14 +3985,14 @@
         </is>
       </c>
       <c r="H74" s="2" t="n">
-        <v>2900</v>
+        <v>2400</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J74" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>38</v>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -4007,12 +4007,12 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Cute Hooded Sweatshirts for Women to Layer and Lounge</t>
+          <t>Plus-Size Graphic Tees: Fit, Print, and Everyday Wear</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>cute hooded sweatshirts for women</t>
+          <t>plus size graphic tees</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -4034,11 +4034,11 @@
         <v>2400</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="J75" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>15</v>
+      </c>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -4053,12 +4053,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Plus-Size Graphic Tees: Fit, Print, and Everyday Wear</t>
+          <t>Cropped Pants for Women: Style Meets Movement</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>plus size graphic tees</t>
+          <t>cropped pants for women</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4077,10 +4077,10 @@
         </is>
       </c>
       <c r="H76" s="2" t="n">
-        <v>2400</v>
+        <v>1900</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="J76" s="8" t="inlineStr">
         <is>
@@ -4099,12 +4099,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Cropped Pants for Women: Style Meets Movement</t>
+          <t>Best Sports Bras for Running: What to Look For</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>cropped pants for women</t>
+          <t>best sports bra for running</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
@@ -4126,7 +4126,7 @@
         <v>1900</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J77" s="8" t="inlineStr">
         <is>
@@ -4145,22 +4145,22 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Best Sports Bras for Running: What to Look For</t>
+          <t>How to Choose Women's Swim Trunks for Comfort</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>best sports bra for running</t>
-        </is>
-      </c>
-      <c r="E78" s="11" t="inlineStr">
-        <is>
-          <t>Sports Bras &amp; Tops</t>
+          <t>swimming trunk for ladies</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
+          <t>Swimwear &amp; Beach</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4169,10 +4169,10 @@
         </is>
       </c>
       <c r="H78" s="2" t="n">
-        <v>1900</v>
+        <v>6600</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>How to Choose Women's Swim Trunks for Comfort</t>
+          <t>High-Waisted Beachwear That Flatters and Stays Put</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>swimming trunk for ladies</t>
+          <t>high waisted beachwear</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -4215,10 +4215,10 @@
         </is>
       </c>
       <c r="H79" s="2" t="n">
-        <v>6600</v>
+        <v>4400</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
@@ -4237,12 +4237,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Beachwear That Flatters and Stays Put</t>
+          <t>One-Piece Swimsuits With Built-In Tummy Control</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>high waisted beachwear</t>
+          <t>1 piece swimsuit tummy control</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
@@ -4261,14 +4261,14 @@
         </is>
       </c>
       <c r="H80" s="2" t="n">
-        <v>4400</v>
+        <v>3600</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="J80" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>13</v>
+      </c>
+      <c r="J80" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -4283,12 +4283,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>One-Piece Swimsuits With Built-In Tummy Control</t>
+          <t>High-Waisted Bathing Suits: Structure Where You Want It</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>1 piece swimsuit tummy control</t>
+          <t>high waisted bathing suits</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -4310,11 +4310,11 @@
         <v>3600</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="J81" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>25</v>
+      </c>
+      <c r="J81" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -6278,9 +6278,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8714,9 +8714,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F90" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -10086,9 +10086,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F139" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -12998,9 +12998,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F243" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F243" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -14118,9 +14118,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F283" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F283" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -15798,9 +15798,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F343" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F343" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
girlievault: keyword workbook with the comparison pieces
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -2995,12 +2995,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Athletic Shorts: Choosing the Right Pair for Every Workout</t>
+          <t>Legging Cuts, Compared: Flare, Straight, Capri and Bike Short</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>athletic shorts</t>
+          <t>flare leggings</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3019,14 +3019,14 @@
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>22200</v>
+        <v>27100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="J53" s="10" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>30</v>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3041,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Straight-Leg Sweatpants: A Buyer's Guide to Fit and Fabric</t>
+          <t>Athletic Shorts: Choosing the Right Pair for Every Workout</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>straight leg sweatpants</t>
+          <t>athletic shorts</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -3065,14 +3065,14 @@
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>12100</v>
+        <v>22200</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J54" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>48</v>
+      </c>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
     </row>
@@ -3087,12 +3087,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>The Best Compression Leggings for Squat-Proof Coverage</t>
+          <t>Straight-Leg Sweatpants: A Buyer's Guide to Fit and Fabric</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>compression leggings</t>
+          <t>straight leg sweatpants</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
         <v>12100</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
@@ -3133,12 +3133,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Workout Shorts: Finding the Right Length and Fit</t>
+          <t>The Best Compression Leggings for Squat-Proof Coverage</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>workout shorts</t>
+          <t>compression leggings</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3157,14 +3157,14 @@
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>9900</v>
+        <v>12100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>24</v>
+      </c>
+      <c r="J56" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Leggings With Pockets: How to Find the Most Functional Pair</t>
+          <t>Workout Shorts: Finding the Right Length and Fit</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>leggings with pockets</t>
+          <t>workout shorts</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -3206,7 +3206,7 @@
         <v>9900</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
@@ -3225,12 +3225,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Yoga Shorts: How to Pick Your Perfect Pair</t>
+          <t>Leggings With Pockets: How to Find the Most Functional Pair</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>yoga shorts</t>
+          <t>leggings with pockets</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
@@ -3249,14 +3249,14 @@
         </is>
       </c>
       <c r="H58" s="2" t="n">
-        <v>6600</v>
+        <v>9900</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="J58" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>39</v>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Fold-Over Leggings: Choosing Your Comfiest Waistband</t>
+          <t>Yoga Shorts: How to Pick Your Perfect Pair</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>fold over leggings</t>
+          <t>yoga shorts</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -3295,10 +3295,10 @@
         </is>
       </c>
       <c r="H59" s="2" t="n">
-        <v>5400</v>
+        <v>6600</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J59" s="8" t="inlineStr">
         <is>
@@ -3317,12 +3317,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Tummy-Control Leggings for Smooth, All-Day Support</t>
+          <t>Fold-Over Leggings: Choosing Your Comfiest Waistband</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>tummy control leggings</t>
+          <t>fold over leggings</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3341,10 +3341,10 @@
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>2900</v>
+        <v>5400</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
@@ -3363,12 +3363,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Legging Shorts: The Length Between Bike Shorts and Leggings</t>
+          <t>Tummy-Control Leggings for Smooth, All-Day Support</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>legging shorts</t>
+          <t>tummy control leggings</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -3390,7 +3390,7 @@
         <v>2900</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>How to Choose Women's Swim Trunks for Comfort</t>
+          <t>One-Piece, Tankini or Bikini: Which Swimsuit Suits You</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>swimming trunk for ladies</t>
+          <t>tankini swimsuit</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4169,10 +4169,10 @@
         </is>
       </c>
       <c r="H78" s="2" t="n">
-        <v>6600</v>
+        <v>22200</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Beachwear That Flatters and Stays Put</t>
+          <t>How to Choose Women's Swim Trunks for Comfort</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>high waisted beachwear</t>
+          <t>swimming trunk for ladies</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -4215,10 +4215,10 @@
         </is>
       </c>
       <c r="H79" s="2" t="n">
-        <v>4400</v>
+        <v>6600</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
@@ -4237,12 +4237,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>One-Piece Swimsuits With Built-In Tummy Control</t>
+          <t>High-Waisted Beachwear That Flatters and Stays Put</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>1 piece swimsuit tummy control</t>
+          <t>high waisted beachwear</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
@@ -4261,14 +4261,14 @@
         </is>
       </c>
       <c r="H80" s="2" t="n">
-        <v>3600</v>
+        <v>4400</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="J80" s="12" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>17</v>
+      </c>
+      <c r="J80" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
     </row>
@@ -4283,12 +4283,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>High-Waisted Bathing Suits: Structure Where You Want It</t>
+          <t>One-Piece Swimsuits With Built-In Tummy Control</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>high waisted bathing suits</t>
+          <t>1 piece swimsuit tummy control</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -4310,11 +4310,11 @@
         <v>3600</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="J81" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>13</v>
+      </c>
+      <c r="J81" s="12" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
     </row>
@@ -6418,9 +6418,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -6670,9 +6670,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -12998,9 +12998,9 @@
           <t>Transactional</t>
         </is>
       </c>
-      <c r="F243" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -15546,9 +15546,9 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="F334" s="7" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -21729,8 +21729,8 @@
     <row r="14" ht="65" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>BoFu (52) — category buying guides for shoppers ready to purchase.
-MoFu (49) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
+          <t>BoFu (50) — category buying guides for shoppers ready to purchase.
+MoFu (51) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
 ToFu (19) — education and styling that builds topical authority and earns citations.
 The MoFu/ToFu weighting is deliberate: those terms are winnable at a young domain and are exactly what AI engines cite when shoppers ask for recommendations.</t>
         </is>

</xml_diff>

<commit_message>
girlievault: keyword-research workbook gains the Plan Changes tab
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Article Plan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Keyword Universe" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Excluded" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Read Me" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Plan Changes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Read Me" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,6 +40,10 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="00333333"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00D10070"/>
       <sz val="16"/>
@@ -52,12 +57,8 @@
       <color rgb="00141414"/>
       <sz val="13"/>
     </font>
-    <font>
-      <color rgb="00333333"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +125,11 @@
         <fgColor rgb="0000A3B4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B3261E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -151,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -168,12 +174,21 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -21647,6 +21662,705 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="64" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Searches</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>REMOVED  (10 articles)</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Workout Sets: The Girlie Vault Guide to Matched Activewear</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>workout sets</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>40500</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Would compete with a page you already rank with</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Swim Shorts for Women: Comfort Meets Coverage</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>swim shorts for women</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>12100</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>No swim shorts in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Swim Skirts: Flattering Coverage for Beach and Pool</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>swim skirt</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>8100</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>No swim skirts in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Tankini Beachwear: Coverage and Confidence in One</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>tankini beachwear</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>6600</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>No tankinis in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>High-Waisted Leggings for All-Day Comfort and Support</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>high waisted leggings</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>6600</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Would compete with a page you already rank with</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Women's Board Shorts: Active Coverage for Sun and Surf</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>womens board shorts</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>5400</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Board shorts are swim shorts under another name, also not stocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Seamless Leggings for a Smooth, Sculpted Fit</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>seamless leggings</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>4400</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>No seamless leggings in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Women's Tracksuit Pants: How to Choose Your Fit</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>tracksuit pants for ladies</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>No tracksuits in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>How to Style Yoga Flare Pants for Any Occasion</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>yoga flare pants outfits</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>No flare cuts in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>The Best Seamless Sports Bras for Everyday Comfort</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>seamless sports bra</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>No seamless bras in the catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>ADDED IN THEIR PLACE  (10 articles)</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="17" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Long-Sleeve Swimsuits: Coverage, Sun Protection, and Fit</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>long sleeve swimsuit</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>6600</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Swim coverage you do sell, and the strongest remaining swim search</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Long Torso Swimsuits: How to Find One That Actually Fits</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>long torso swimsuits</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>4400</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>A fit problem your one-pieces answer directly</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Spring Break Swimwear: What to Pack and How to Choose</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>spring break swimwear</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>4400</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Seasonal demand across your whole swim line</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Full-Coverage Swimsuits: Comfort In and Out of the Water</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>full coverage swimsuit</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Coverage without the shapewear framing you asked us to avoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Women's Jogger Sets: How to Pick One You Will Live In</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>female jogger set</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Matching sets are a category you actually stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Going-Out Sets: Matching Pieces That Work Past the Gym</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>going out sets</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Extends matching sets past the gym, which is the lifestyle positioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Gym Hoodies: Choosing One for Warm-Ups and Cool-Downs</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>gym hoodies</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Hoodies are in the catalogue and had no article</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Bikini Tops for a Smaller Bust: How to Find Your Fit</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>bikinis to suit small bust</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>A fit question your bikini tops answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Plus-Size Graphic Tees: Fit, Print, and Everyday Wear</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>plus size graphic tees</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Graphic tees you sell, including the Pledge line</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Leopard Print Leggings: How to Wear a Bold Pattern</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>leopard print leggings</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Bold print is the brand's whole identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>KEPT, NEW ANGLE  (3 articles)</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>was:  The Girlie Vault Guide to Flare Leggings
+now:  Legging Cuts, Compared: Flare, Straight, Capri and Bike Short</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>flare leggings</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>27100</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>You do not sell flare, but it is the largest search we found. A cut comparison catches the shopper while she is still choosing, and three of the four cuts it covers are yours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>was:  Tankini Swimsuits: How to Find Your Perfect Fit
+now:  One-Piece, Tankini or Bikini: Which Swimsuit Suits You</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>tankini swimsuit</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>22200</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Same reasoning. A format comparison earns the search without promising a tankini, and your one-piece and bikini lines are the answer it gives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>was:  Plus-Size Workout Clothes for Confident Movement
+now:  Plus-Size Activewear That Moves: A Fit and Fabric Guide</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>plus size workout clothes</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>6600</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Retitled only. The original sat too close to an article you already have.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="108" customHeight="1">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
+On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
+The two largest searches we would otherwise have lost, 55,900 between them, are kept as the comparison articles in the third block rather than dropped.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A29:F29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -21654,45 +22368,46 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Girlie Vault — Keyword Research Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Companion to your SEO Growth Roadmap. Built from SEMrush Keyword Strategy Builder + Keyword Gap (US).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>What's in this workbook</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="65" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>1. Article Plan        — the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD).
 2. Keyword Universe    — the broader research surfaced from SEMrush; keywords already in the plan are flagged 'Yes (planned)', the rest are 'Overflow' opportunities for later months.
 3. Excluded            — high-volume keywords we intentionally left out, with the reason for each.
-4. Read Me             — this tab.</t>
+4. Plan Changes        — every article swapped or re-angled since the plan you approved in July, with the old topic, the new one, and why.
+5. Read Me             — this tab.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>How to read difficulty (KD)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>KD is SEMrush's 0-100 ranking-difficulty score. We front-load easy wins for a young domain:
   Very Easy (&lt;15) · Easy (15-29) · Moderate (30-44) · Hard (45+).
@@ -21701,14 +22416,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>The six content pillars</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Leggings &amp; Bottoms      — your largest commercial cluster (leggings with pockets, seamless, compression, biker shorts).
 Swimwear &amp; Beach        — one-piece, bikini sets, prints and patterns, rash guards.
@@ -21720,14 +22435,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Funnel philosophy</t>
         </is>
       </c>
     </row>
     <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>BoFu (50) — category buying guides for shoppers ready to purchase.
 MoFu (51) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
@@ -21737,14 +22452,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>What we excluded, and why</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>See the 'Excluded' tab for the full list. The big categories:
   Menswear / couples        — off-audience for a women's brand.
@@ -21757,28 +22472,28 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>Working titles</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Headlines in the Article Plan are working titles: the keyword, angle and funnel stage are locked, but the exact wording is finalized at production with an SEO title-lock pass. Your input on titles is welcome.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Approve the plan and ClusterMagic begins the Month 1 batch. Articles are entity-rich, internally linked, schema-marked, and shipped to your store as drafts for review. The Reddit/AEO layer runs alongside to start earning brand mentions in AI answers.</t>
         </is>

</xml_diff>

<commit_message>
girlievault: workbook gains the existing-pages proposal block
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -58,7 +62,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +134,11 @@
         <fgColor rgb="00B3261E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A73E8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -157,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -183,12 +192,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -21662,7 +21674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -22338,18 +22350,149 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="108" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>YOUR EXISTING BLOG PAGES  (proposed, nothing changes without your OK)</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="22" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>Google, last 90 days</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>What we propose and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Finding the Best Leggings for Thick Thighs: A Guide to ...</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>3,558 shown / 22 clicks</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting your OK</t>
+        </is>
+      </c>
+      <c r="F30" s="20" t="inlineStr">
+        <is>
+          <t>New title and description in Google only; the article itself stays as is. The page already ranks on page 1, the current headline undersells it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>How to Wear Leggings for Any Occasion and Feel Absolutely Confident</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>507 shown / 0 clicks</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting your OK</t>
+        </is>
+      </c>
+      <c r="F31" s="20" t="inlineStr">
+        <is>
+          <t>Full rewrite built around the questions people actually type, like 'how do you wear high waisted leggings'. Sits on page 2 today with zero clicks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Finding the Best High Waisted Leggings for You</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>168 shown / 0 clicks</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting your OK</t>
+        </is>
+      </c>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>Merge its best content into How to Wear Leggings and redirect the old address there. The two pages currently compete for the same searches, so Google shows neither one well. Every old link keeps working.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Your Guide to the Best Matching Workout Sets</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>94 shown / 0 clicks</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Left as is for now</t>
+        </is>
+      </c>
+      <c r="F33" s="20" t="inlineStr">
+        <is>
+          <t>Nothing for now. That search is dominated by big-brand store pages; we will revisit once the first two show movement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="138" customHeight="1">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
 On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
-The two largest searches we would otherwise have lost, 55,900 between them, are kept as the comparison articles in the third block rather than dropped.</t>
+The two largest searches we would otherwise have lost, 55,900 between them, are kept as the comparison articles in the third block rather than dropped.
+The last block is different: those pages already exist on your blog, written before we came on board. Nothing there changes until you give the OK, and the workout sets page is staying as it is either way.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A35:F35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22368,46 +22511,46 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Girlie Vault — Keyword Research Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Companion to your SEO Growth Roadmap. Built from SEMrush Keyword Strategy Builder + Keyword Gap (US).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>What's in this workbook</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>1. Article Plan        — the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD).
-2. Keyword Universe    — the broader research surfaced from SEMrush; keywords already in the plan are flagged 'Yes (planned)', the rest are 'Overflow' opportunities for later months.
-3. Excluded            — high-volume keywords we intentionally left out, with the reason for each.
-4. Plan Changes        — every article swapped or re-angled since the plan you approved in July, with the old topic, the new one, and why.
-5. Read Me             — this tab.</t>
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD).
+2. Keyword Universe    · the broader research surfaced from SEMrush; keywords already in the plan are flagged 'Yes (planned)', the rest are 'Overflow' opportunities for later months.
+3. Excluded            · high-volume keywords we intentionally left out, with the reason for each.
+4. Plan Changes        · every article swapped or re-angled since the plan you approved in July, plus the four pages that already exist on your blog and what we have proposed for each.
+5. Read Me             · this tab.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>How to read difficulty (KD)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>KD is SEMrush's 0-100 ranking-difficulty score. We front-load easy wins for a young domain:
   Very Easy (&lt;15) · Easy (15-29) · Moderate (30-44) · Hard (45+).
@@ -22416,84 +22559,84 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>The six content pillars</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>Leggings &amp; Bottoms      — your largest commercial cluster (leggings with pockets, seamless, compression, biker shorts).
-Swimwear &amp; Beach        — one-piece, bikini sets, prints and patterns, rash guards.
-Sports Bras &amp; Tops      — sports bras, workout tops, crop tops (sports bras only, not lingerie).
-Matching Sets &amp; Outfits — matching workout sets, gym sets, outfit styling.
-Activewear Style &amp; Education — how-to, styling, fabric and buying guides (top-funnel discovery + AI citations).
-Brand, Give-Back &amp; Community — founder story, Take the Pledge / City Harvest, Give Back Girls, women-empowerment (branded trust + AI naming).</t>
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Leggings &amp; Bottoms      · your largest commercial cluster (leggings with pockets, seamless, compression, biker shorts).
+Swimwear &amp; Beach        · one-piece, bikini sets, prints and patterns, rash guards.
+Sports Bras &amp; Tops      · sports bras, workout tops, crop tops (sports bras only, not lingerie).
+Matching Sets &amp; Outfits · matching workout sets, gym sets, outfit styling.
+Activewear Style &amp; Education · how-to, styling, fabric and buying guides (top-funnel discovery + AI citations).
+Brand, Give-Back &amp; Community · founder story, Take the Pledge / City Harvest, Give Back Girls, women-empowerment (branded trust + AI naming).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Funnel philosophy</t>
         </is>
       </c>
     </row>
     <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>BoFu (50) — category buying guides for shoppers ready to purchase.
-MoFu (51) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
-ToFu (19) — education and styling that builds topical authority and earns citations.
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>BoFu (50) · category buying guides for shoppers ready to purchase.
+MoFu (51) · best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
+ToFu (19) · education and styling that builds topical authority and earns citations.
 The MoFu/ToFu weighting is deliberate: those terms are winnable at a young domain and are exactly what AI engines cite when shoppers ask for recommendations.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>What we excluded, and why</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>See the 'Excluded' tab for the full list. The big categories:
-  Menswear / couples        — off-audience for a women's brand.
-  Everyday / lingerie bras   — you sell sports bras, not lingerie.
-  Wrong audience (over 50)   — outside the brand's core shopper.
-  Off-brand swim (thong/micro)— off-tone for the empowerment/give-back positioning.
-  Competitor brand terms      — 'lululemon leggings' can't be won with your content.
-  Non-catalog / off-vertical  — socks, sewing patterns, costumes.</t>
+  Menswear / couples        · off-audience for a women's brand.
+  Everyday / lingerie bras   · you sell sports bras, not lingerie.
+  Wrong audience (over 50)   · outside the brand's core shopper.
+  Off-brand swim (thong/micro)· off-tone for the empowerment/give-back positioning.
+  Competitor brand terms      · 'lululemon leggings' can't be won with your content.
+  Non-catalog / off-vertical  · socks, sewing patterns, costumes.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Working titles</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Headlines in the Article Plan are working titles: the keyword, angle and funnel stage are locked, but the exact wording is finalized at production with an SEO title-lock pass. Your input on titles is welcome.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Approve the plan and ClusterMagic begins the Month 1 batch. Articles are entity-rich, internally linked, schema-marked, and shipped to your store as drafts for review. The Reddit/AEO layer runs alongside to start earning brand mentions in AI answers.</t>
         </is>

</xml_diff>

<commit_message>
girlievault: proposal block trimmed to the three actionable pages
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21674,7 +21674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -22456,43 +22456,19 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="40" customHeight="1">
-      <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Your Guide to the Best Matching Workout Sets</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>94 shown / 0 clicks</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Left as is for now</t>
-        </is>
-      </c>
-      <c r="F33" s="20" t="inlineStr">
-        <is>
-          <t>Nothing for now. That search is dominated by big-brand store pages; we will revisit once the first two show movement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="138" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
+    <row r="34" ht="138" customHeight="1">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
 On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
 The two largest searches we would otherwise have lost, 55,900 between them, are kept as the comparison articles in the third block rather than dropped.
-The last block is different: those pages already exist on your blog, written before we came on board. Nothing there changes until you give the OK, and the workout sets page is staying as it is either way.</t>
+The last block is different: those pages already exist on your blog, written before we came on board. Nothing there changes until you give the OK.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A34:F34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
girlievault: workbook statuses match the email posture
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21681,7 +21681,7 @@
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="64" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -22353,7 +22353,7 @@
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>YOUR EXISTING BLOG PAGES  (proposed, nothing changes without your OK)</t>
+          <t>YOUR EXISTING BLOG PAGES  (nothing goes live without your review)</t>
         </is>
       </c>
       <c r="B28" s="22" t="n"/>
@@ -22399,7 +22399,7 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Awaiting your OK</t>
+          <t>Going ahead</t>
         </is>
       </c>
       <c r="F30" s="20" t="inlineStr">
@@ -22423,7 +22423,7 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Awaiting your OK</t>
+          <t>Going ahead</t>
         </is>
       </c>
       <c r="F31" s="20" t="inlineStr">
@@ -22462,7 +22462,7 @@
           <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
 On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
 The two largest searches we would otherwise have lost, 55,900 between them, are kept as the comparison articles in the third block rather than dropped.
-The last block is different: those pages already exist on your blog, written before we came on board. Nothing there changes until you give the OK.</t>
+The last block is different: those pages already exist on your blog, written before we came on board. The first two go ahead under the go-ahead from your last email, and you review each as a draft before it goes live. The page merge is the one thing waiting on your explicit OK.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
girlievault: workbook highlights changed rows inline
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,16 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009A6E00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E8E3E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -62,7 +72,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -111,7 +121,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF6E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E8743C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -166,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -179,28 +199,32 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -566,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -579,6 +603,7 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -632,6 +657,11 @@
           <t>Difficulty</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -678,6 +708,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -724,6 +755,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -770,6 +802,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -816,6 +849,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -862,6 +896,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -912,6 +947,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -962,6 +998,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1012,6 +1049,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1062,6 +1100,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1108,6 +1147,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1154,6 +1194,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1200,6 +1241,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1246,6 +1288,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1292,6 +1335,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1338,6 +1382,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1384,6 +1429,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1430,22 +1476,23 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Plus-Size Activewear That Moves: A Fit and Fabric Guide</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>plus size workout clothes</t>
         </is>
@@ -1455,25 +1502,30 @@
           <t>Matching Sets &amp; Outfits</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n">
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="n">
         <v>6600</v>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="I19" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="J19" s="10" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
+        </is>
+      </c>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>New angle</t>
         </is>
       </c>
     </row>
@@ -1522,6 +1574,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1563,27 +1616,28 @@
       <c r="I21" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="J21" s="10" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="13" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>Women's Jogger Sets: How to Pick One You Will Live In</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>female jogger set</t>
         </is>
@@ -1593,25 +1647,30 @@
           <t>Matching Sets &amp; Outfits</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>BoFu</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="n">
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="n">
         <v>3600</v>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I22" s="13" t="n">
         <v>28</v>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1655,11 +1714,12 @@
       <c r="I23" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="J23" s="10" t="inlineStr">
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1680,7 +1740,7 @@
           <t>cropped tank top</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -1701,11 +1761,12 @@
       <c r="I24" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J24" s="12" t="inlineStr">
+      <c r="J24" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1726,7 +1787,7 @@
           <t>high sports bra support</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -1752,6 +1813,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1772,7 +1834,7 @@
           <t>plus size sports bra</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -1798,6 +1860,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1818,7 +1881,7 @@
           <t>yellow tank top</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -1844,6 +1907,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1864,7 +1928,7 @@
           <t>cotton sports bra</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -1890,50 +1954,56 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="13" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>Gym Hoodies: Choosing One for Warm-Ups and Cool-Downs</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>gym hoodies</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="n">
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n">
         <v>2900</v>
       </c>
-      <c r="I29" s="2" t="n">
+      <c r="I29" s="13" t="n">
         <v>16</v>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K29" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1956,7 +2026,7 @@
           <t>string bikini</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -1982,6 +2052,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2002,7 +2073,7 @@
           <t>high waisted bikini</t>
         </is>
       </c>
-      <c r="E31" s="13" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -2028,6 +2099,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2048,7 +2120,7 @@
           <t>tummy control swimsuit</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -2074,6 +2146,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2094,7 +2167,7 @@
           <t>black one piece swimsuit</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -2120,6 +2193,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2140,7 +2214,7 @@
           <t>bikini bottoms</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -2166,6 +2240,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2186,7 +2261,7 @@
           <t>high waisted bikini bottoms</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -2212,50 +2287,56 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="13" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="13" t="inlineStr">
         <is>
           <t>Long-Sleeve Swimsuits: Coverage, Sun Protection, and Fit</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>long sleeve swimsuit</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="n">
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="n">
         <v>6600</v>
       </c>
-      <c r="I36" s="2" t="n">
+      <c r="I36" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="J36" s="12" t="inlineStr">
+      <c r="J36" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="K36" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2359,7 @@
           <t>two piece swimming costumes for ladies</t>
         </is>
       </c>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -2304,137 +2385,148 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="13" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="13" t="inlineStr">
         <is>
           <t>Long Torso Swimsuits: How to Find One That Actually Fits</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>long torso swimsuits</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F38" s="13" t="inlineStr">
         <is>
           <t>BoFu</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="n">
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="n">
         <v>4400</v>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="I38" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="J38" s="12" t="inlineStr">
+      <c r="J38" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="13" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>Spring Break Swimwear: What to Pack and How to Choose</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>spring break swimwear</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F39" s="13" t="inlineStr">
         <is>
           <t>ToFu</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="n">
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="n">
         <v>4400</v>
       </c>
-      <c r="I39" s="2" t="n">
+      <c r="I39" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="J39" s="12" t="inlineStr">
+      <c r="J39" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
+      <c r="K39" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="13" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="13" t="inlineStr">
         <is>
           <t>Full-Coverage Swimsuits: Comfort In and Out of the Water</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
         <is>
           <t>full coverage swimsuit</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E40" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F40" s="13" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="n">
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="n">
         <v>3600</v>
       </c>
-      <c r="I40" s="2" t="n">
+      <c r="I40" s="13" t="n">
         <v>16</v>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -2442,50 +2534,60 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K40" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>Bikini Tops for a Smaller Bust: How to Find Your Fit</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>bikinis to suit small bust</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F41" s="13" t="inlineStr">
         <is>
           <t>BoFu</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="n">
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="n">
         <v>2900</v>
       </c>
-      <c r="I41" s="2" t="n">
+      <c r="I41" s="13" t="n">
         <v>15</v>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K41" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2529,11 +2631,12 @@
       <c r="I42" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="J42" s="10" t="inlineStr">
+      <c r="J42" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2580,6 +2683,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2621,11 +2725,12 @@
       <c r="I44" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J44" s="10" t="inlineStr">
+      <c r="J44" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2672,6 +2777,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2718,6 +2824,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2768,6 +2875,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2818,6 +2926,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2868,6 +2977,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2918,6 +3028,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2964,6 +3075,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -3010,22 +3122,23 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>Legging Cuts, Compared: Flare, Straight, Capri and Bike Short</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>flare leggings</t>
         </is>
@@ -3035,25 +3148,30 @@
           <t>Leggings &amp; Bottoms</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F53" s="10" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="n">
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H53" s="10" t="n">
         <v>27100</v>
       </c>
-      <c r="I53" s="2" t="n">
+      <c r="I53" s="10" t="n">
         <v>30</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
           <t>Moderate</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>New angle</t>
         </is>
       </c>
     </row>
@@ -3097,11 +3215,12 @@
       <c r="I54" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="J54" s="10" t="inlineStr">
+      <c r="J54" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3148,6 +3267,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3194,6 +3314,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -3240,6 +3361,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3286,6 +3408,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3332,6 +3455,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3378,6 +3502,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3424,6 +3549,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3470,6 +3596,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3516,6 +3643,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3562,6 +3690,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3608,22 +3737,23 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="13" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="13" t="inlineStr">
         <is>
           <t>Going-Out Sets: Matching Pieces That Work Past the Gym</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="13" t="inlineStr">
         <is>
           <t>going out sets</t>
         </is>
@@ -3633,25 +3763,30 @@
           <t>Matching Sets &amp; Outfits</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" s="13" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="n">
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H66" s="13" t="n">
         <v>3600</v>
       </c>
-      <c r="I66" s="2" t="n">
+      <c r="I66" s="13" t="n">
         <v>21</v>
       </c>
       <c r="J66" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K66" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -3700,6 +3835,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3746,6 +3882,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3766,7 +3903,7 @@
           <t>racerback bra</t>
         </is>
       </c>
-      <c r="E69" s="11" t="inlineStr">
+      <c r="E69" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -3792,6 +3929,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3812,7 +3950,7 @@
           <t>tank top with built in bra</t>
         </is>
       </c>
-      <c r="E70" s="11" t="inlineStr">
+      <c r="E70" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -3838,6 +3976,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3858,7 +3997,7 @@
           <t>racerback tank</t>
         </is>
       </c>
-      <c r="E71" s="11" t="inlineStr">
+      <c r="E71" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -3884,6 +4023,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -3904,7 +4044,7 @@
           <t>push up sports bra</t>
         </is>
       </c>
-      <c r="E72" s="11" t="inlineStr">
+      <c r="E72" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -3930,6 +4070,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3950,7 +4091,7 @@
           <t>compression sports bra</t>
         </is>
       </c>
-      <c r="E73" s="11" t="inlineStr">
+      <c r="E73" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -3976,6 +4117,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3996,7 +4138,7 @@
           <t>cute hooded sweatshirts for women</t>
         </is>
       </c>
-      <c r="E74" s="11" t="inlineStr">
+      <c r="E74" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -4022,50 +4164,56 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="13" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B75" s="13" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C75" s="13" t="inlineStr">
         <is>
           <t>Plus-Size Graphic Tees: Fit, Print, and Everyday Wear</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D75" s="13" t="inlineStr">
         <is>
           <t>plus size graphic tees</t>
         </is>
       </c>
-      <c r="E75" s="11" t="inlineStr">
+      <c r="E75" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F75" s="13" t="inlineStr">
         <is>
           <t>BoFu</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="n">
+      <c r="G75" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H75" s="13" t="n">
         <v>2400</v>
       </c>
-      <c r="I75" s="2" t="n">
+      <c r="I75" s="13" t="n">
         <v>15</v>
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K75" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4236,7 @@
           <t>cropped pants for women</t>
         </is>
       </c>
-      <c r="E76" s="11" t="inlineStr">
+      <c r="E76" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -4114,6 +4262,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -4134,7 +4283,7 @@
           <t>best sports bra for running</t>
         </is>
       </c>
-      <c r="E77" s="11" t="inlineStr">
+      <c r="E77" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -4160,50 +4309,56 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B78" s="10" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C78" s="10" t="inlineStr">
         <is>
           <t>One-Piece, Tankini or Bikini: Which Swimsuit Suits You</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D78" s="10" t="inlineStr">
         <is>
           <t>tankini swimsuit</t>
         </is>
       </c>
-      <c r="E78" s="13" t="inlineStr">
+      <c r="E78" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F78" s="10" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="n">
+      <c r="G78" s="10" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H78" s="10" t="n">
         <v>22200</v>
       </c>
-      <c r="I78" s="2" t="n">
+      <c r="I78" s="10" t="n">
         <v>28</v>
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K78" s="12" t="inlineStr">
+        <is>
+          <t>New angle</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4381,7 @@
           <t>swimming trunk for ladies</t>
         </is>
       </c>
-      <c r="E79" s="13" t="inlineStr">
+      <c r="E79" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -4252,6 +4407,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -4272,7 +4428,7 @@
           <t>high waisted beachwear</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
+      <c r="E80" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -4298,6 +4454,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -4318,7 +4475,7 @@
           <t>1 piece swimsuit tummy control</t>
         </is>
       </c>
-      <c r="E81" s="13" t="inlineStr">
+      <c r="E81" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -4339,11 +4496,12 @@
       <c r="I81" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J81" s="12" t="inlineStr">
+      <c r="J81" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
+      <c r="K81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -4390,6 +4548,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -4436,6 +4595,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4482,6 +4642,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4523,11 +4684,12 @@
       <c r="I85" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="J85" s="10" t="inlineStr">
+      <c r="J85" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4574,6 +4736,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -4620,6 +4783,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4666,6 +4830,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -4712,6 +4877,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -4762,6 +4928,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -4812,6 +4979,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -4862,6 +5030,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -4912,6 +5081,7 @@
           <t>Brand</t>
         </is>
       </c>
+      <c r="K93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -4953,11 +5123,12 @@
       <c r="I94" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J94" s="10" t="inlineStr">
+      <c r="J94" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -5004,6 +5175,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -5050,6 +5222,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -5096,6 +5269,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -5137,11 +5311,12 @@
       <c r="I98" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="J98" s="10" t="inlineStr">
+      <c r="J98" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -5188,6 +5363,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -5234,6 +5410,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -5280,6 +5457,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -5326,22 +5504,23 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="13" t="n">
         <v>102</v>
       </c>
-      <c r="B103" s="2" t="inlineStr">
+      <c r="B103" s="13" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C103" s="13" t="inlineStr">
         <is>
           <t>Leopard Print Leggings: How to Wear a Bold Pattern</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D103" s="13" t="inlineStr">
         <is>
           <t>leopard print leggings</t>
         </is>
@@ -5351,25 +5530,30 @@
           <t>Leggings &amp; Bottoms</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr">
+      <c r="F103" s="13" t="inlineStr">
         <is>
           <t>MoFu</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="H103" s="2" t="n">
+      <c r="G103" s="13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H103" s="13" t="n">
         <v>1900</v>
       </c>
-      <c r="I103" s="2" t="n">
+      <c r="I103" s="13" t="n">
         <v>24</v>
       </c>
       <c r="J103" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
+        </is>
+      </c>
+      <c r="K103" s="14" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -5418,6 +5602,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -5464,6 +5649,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -5510,6 +5696,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -5551,11 +5738,12 @@
       <c r="I107" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J107" s="12" t="inlineStr">
+      <c r="J107" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
+      <c r="K107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -5576,7 +5764,7 @@
           <t>pink tank top</t>
         </is>
       </c>
-      <c r="E108" s="11" t="inlineStr">
+      <c r="E108" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -5602,6 +5790,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -5622,7 +5811,7 @@
           <t>white sports bra</t>
         </is>
       </c>
-      <c r="E109" s="11" t="inlineStr">
+      <c r="E109" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -5648,6 +5837,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -5668,7 +5858,7 @@
           <t>workout tank tops</t>
         </is>
       </c>
-      <c r="E110" s="11" t="inlineStr">
+      <c r="E110" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -5694,6 +5884,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -5714,7 +5905,7 @@
           <t>best sports bra for large breasts</t>
         </is>
       </c>
-      <c r="E111" s="11" t="inlineStr">
+      <c r="E111" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -5740,6 +5931,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -5760,7 +5952,7 @@
           <t>athletic jacket</t>
         </is>
       </c>
-      <c r="E112" s="11" t="inlineStr">
+      <c r="E112" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -5786,6 +5978,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -5806,7 +5999,7 @@
           <t>workout tanks for women</t>
         </is>
       </c>
-      <c r="E113" s="11" t="inlineStr">
+      <c r="E113" s="15" t="inlineStr">
         <is>
           <t>Sports Bras &amp; Tops</t>
         </is>
@@ -5832,6 +6025,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -5852,7 +6046,7 @@
           <t>one piece swimsuit</t>
         </is>
       </c>
-      <c r="E114" s="13" t="inlineStr">
+      <c r="E114" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -5878,6 +6072,7 @@
           <t>Moderate</t>
         </is>
       </c>
+      <c r="K114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -5898,7 +6093,7 @@
           <t>dresses for bathing suits</t>
         </is>
       </c>
-      <c r="E115" s="13" t="inlineStr">
+      <c r="E115" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -5924,6 +6119,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K115" s="2" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -5944,7 +6140,7 @@
           <t>triangle bikini top</t>
         </is>
       </c>
-      <c r="E116" s="13" t="inlineStr">
+      <c r="E116" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -5970,6 +6166,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -5990,7 +6187,7 @@
           <t>best swimsuits for ladies</t>
         </is>
       </c>
-      <c r="E117" s="13" t="inlineStr">
+      <c r="E117" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -6011,11 +6208,12 @@
       <c r="I117" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J117" s="10" t="inlineStr">
+      <c r="J117" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
+      <c r="K117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -6036,7 +6234,7 @@
           <t>high waisted swimsuit</t>
         </is>
       </c>
-      <c r="E118" s="13" t="inlineStr">
+      <c r="E118" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -6062,6 +6260,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -6082,7 +6281,7 @@
           <t>swim shirts for women</t>
         </is>
       </c>
-      <c r="E119" s="13" t="inlineStr">
+      <c r="E119" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -6108,6 +6307,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -6128,7 +6328,7 @@
           <t>tummy control bikini</t>
         </is>
       </c>
-      <c r="E120" s="13" t="inlineStr">
+      <c r="E120" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -6149,11 +6349,12 @@
       <c r="I120" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J120" s="12" t="inlineStr">
+      <c r="J120" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
+      <c r="K120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -6174,7 +6375,7 @@
           <t>swim tops for women</t>
         </is>
       </c>
-      <c r="E121" s="13" t="inlineStr">
+      <c r="E121" s="17" t="inlineStr">
         <is>
           <t>Swimwear &amp; Beach</t>
         </is>
@@ -6200,6 +6401,7 @@
           <t>Easy</t>
         </is>
       </c>
+      <c r="K121" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6351,7 +6553,7 @@
       <c r="C5" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -6631,7 +6833,7 @@
       <c r="C15" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -6715,7 +6917,7 @@
       <c r="C18" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -6743,7 +6945,7 @@
       <c r="C19" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -7107,7 +7309,7 @@
       <c r="C32" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -7275,7 +7477,7 @@
       <c r="C38" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D38" s="10" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -7499,7 +7701,7 @@
       <c r="C46" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="D46" s="10" t="inlineStr">
+      <c r="D46" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -7583,7 +7785,7 @@
       <c r="C49" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="D49" s="10" t="inlineStr">
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -7723,7 +7925,7 @@
       <c r="C54" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="D54" s="10" t="inlineStr">
+      <c r="D54" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -7891,7 +8093,7 @@
       <c r="C60" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8087,7 +8289,7 @@
       <c r="C67" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="D67" s="10" t="inlineStr">
+      <c r="D67" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8115,7 +8317,7 @@
       <c r="C68" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="D68" s="10" t="inlineStr">
+      <c r="D68" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8227,7 +8429,7 @@
       <c r="C72" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="D72" s="10" t="inlineStr">
+      <c r="D72" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8255,7 +8457,7 @@
       <c r="C73" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D73" s="10" t="inlineStr">
+      <c r="D73" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8479,7 +8681,7 @@
       <c r="C81" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D81" s="10" t="inlineStr">
+      <c r="D81" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8507,7 +8709,7 @@
       <c r="C82" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D82" s="10" t="inlineStr">
+      <c r="D82" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8535,7 +8737,7 @@
       <c r="C83" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D83" s="10" t="inlineStr">
+      <c r="D83" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8563,7 +8765,7 @@
       <c r="C84" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D84" s="10" t="inlineStr">
+      <c r="D84" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8843,7 +9045,7 @@
       <c r="C94" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D94" s="10" t="inlineStr">
+      <c r="D94" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -8955,7 +9157,7 @@
       <c r="C98" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="D98" s="10" t="inlineStr">
+      <c r="D98" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9095,7 +9297,7 @@
       <c r="C103" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="D103" s="10" t="inlineStr">
+      <c r="D103" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9179,7 +9381,7 @@
       <c r="C106" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="D106" s="10" t="inlineStr">
+      <c r="D106" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9235,7 +9437,7 @@
       <c r="C108" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D108" s="10" t="inlineStr">
+      <c r="D108" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9263,7 +9465,7 @@
       <c r="C109" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="D109" s="10" t="inlineStr">
+      <c r="D109" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9347,7 +9549,7 @@
       <c r="C112" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="D112" s="10" t="inlineStr">
+      <c r="D112" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9375,7 +9577,7 @@
       <c r="C113" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="D113" s="10" t="inlineStr">
+      <c r="D113" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9459,7 +9661,7 @@
       <c r="C116" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D116" s="12" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -9543,7 +9745,7 @@
       <c r="C119" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="D119" s="10" t="inlineStr">
+      <c r="D119" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9599,7 +9801,7 @@
       <c r="C121" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D121" s="10" t="inlineStr">
+      <c r="D121" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9627,7 +9829,7 @@
       <c r="C122" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="D122" s="10" t="inlineStr">
+      <c r="D122" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -9655,7 +9857,7 @@
       <c r="C123" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D123" s="12" t="inlineStr">
+      <c r="D123" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -9683,7 +9885,7 @@
       <c r="C124" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D124" s="12" t="inlineStr">
+      <c r="D124" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -10019,7 +10221,7 @@
       <c r="C136" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="D136" s="10" t="inlineStr">
+      <c r="D136" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10047,7 +10249,7 @@
       <c r="C137" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="D137" s="10" t="inlineStr">
+      <c r="D137" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10243,7 +10445,7 @@
       <c r="C144" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D144" s="12" t="inlineStr">
+      <c r="D144" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -10383,7 +10585,7 @@
       <c r="C149" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="D149" s="10" t="inlineStr">
+      <c r="D149" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10439,7 +10641,7 @@
       <c r="C151" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="D151" s="10" t="inlineStr">
+      <c r="D151" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10467,7 +10669,7 @@
       <c r="C152" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="D152" s="10" t="inlineStr">
+      <c r="D152" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10495,7 +10697,7 @@
       <c r="C153" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="D153" s="10" t="inlineStr">
+      <c r="D153" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10747,7 +10949,7 @@
       <c r="C162" s="2" t="n">
         <v>92</v>
       </c>
-      <c r="D162" s="10" t="inlineStr">
+      <c r="D162" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -10943,7 +11145,7 @@
       <c r="C169" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D169" s="12" t="inlineStr">
+      <c r="D169" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -11055,7 +11257,7 @@
       <c r="C173" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D173" s="12" t="inlineStr">
+      <c r="D173" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -11083,7 +11285,7 @@
       <c r="C174" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="D174" s="10" t="inlineStr">
+      <c r="D174" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -11279,7 +11481,7 @@
       <c r="C181" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D181" s="12" t="inlineStr">
+      <c r="D181" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -11391,7 +11593,7 @@
       <c r="C185" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D185" s="12" t="inlineStr">
+      <c r="D185" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -11587,7 +11789,7 @@
       <c r="C192" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D192" s="12" t="inlineStr">
+      <c r="D192" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -11643,7 +11845,7 @@
       <c r="C194" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D194" s="10" t="inlineStr">
+      <c r="D194" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -11951,7 +12153,7 @@
       <c r="C205" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="D205" s="10" t="inlineStr">
+      <c r="D205" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -11979,7 +12181,7 @@
       <c r="C206" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="D206" s="10" t="inlineStr">
+      <c r="D206" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12007,7 +12209,7 @@
       <c r="C207" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D207" s="10" t="inlineStr">
+      <c r="D207" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12063,7 +12265,7 @@
       <c r="C209" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D209" s="10" t="inlineStr">
+      <c r="D209" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12175,7 +12377,7 @@
       <c r="C213" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="D213" s="10" t="inlineStr">
+      <c r="D213" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12203,7 +12405,7 @@
       <c r="C214" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="D214" s="10" t="inlineStr">
+      <c r="D214" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12231,7 +12433,7 @@
       <c r="C215" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D215" s="12" t="inlineStr">
+      <c r="D215" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -12259,7 +12461,7 @@
       <c r="C216" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D216" s="10" t="inlineStr">
+      <c r="D216" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12315,7 +12517,7 @@
       <c r="C218" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="D218" s="10" t="inlineStr">
+      <c r="D218" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12427,7 +12629,7 @@
       <c r="C222" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D222" s="10" t="inlineStr">
+      <c r="D222" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12539,7 +12741,7 @@
       <c r="C226" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="D226" s="10" t="inlineStr">
+      <c r="D226" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -12987,7 +13189,7 @@
       <c r="C242" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D242" s="10" t="inlineStr">
+      <c r="D242" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -13127,7 +13329,7 @@
       <c r="C247" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="D247" s="10" t="inlineStr">
+      <c r="D247" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -13435,7 +13637,7 @@
       <c r="C258" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D258" s="12" t="inlineStr">
+      <c r="D258" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -13491,7 +13693,7 @@
       <c r="C260" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D260" s="10" t="inlineStr">
+      <c r="D260" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -13967,7 +14169,7 @@
       <c r="C277" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="D277" s="10" t="inlineStr">
+      <c r="D277" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -13995,7 +14197,7 @@
       <c r="C278" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="D278" s="10" t="inlineStr">
+      <c r="D278" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -14107,7 +14309,7 @@
       <c r="C282" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="D282" s="10" t="inlineStr">
+      <c r="D282" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -14415,7 +14617,7 @@
       <c r="C293" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D293" s="12" t="inlineStr">
+      <c r="D293" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -14443,7 +14645,7 @@
       <c r="C294" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="D294" s="12" t="inlineStr">
+      <c r="D294" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -14527,7 +14729,7 @@
       <c r="C297" s="2" t="n">
         <v>96</v>
       </c>
-      <c r="D297" s="10" t="inlineStr">
+      <c r="D297" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -14639,7 +14841,7 @@
       <c r="C301" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="D301" s="10" t="inlineStr">
+      <c r="D301" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -14723,7 +14925,7 @@
       <c r="C304" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D304" s="12" t="inlineStr">
+      <c r="D304" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -14975,7 +15177,7 @@
       <c r="C313" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="D313" s="12" t="inlineStr">
+      <c r="D313" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -15535,7 +15737,7 @@
       <c r="C333" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="D333" s="10" t="inlineStr">
+      <c r="D333" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -15899,7 +16101,7 @@
       <c r="C346" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="D346" s="10" t="inlineStr">
+      <c r="D346" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -16235,7 +16437,7 @@
       <c r="C358" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D358" s="12" t="inlineStr">
+      <c r="D358" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -16459,7 +16661,7 @@
       <c r="C366" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D366" s="10" t="inlineStr">
+      <c r="D366" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -16487,7 +16689,7 @@
       <c r="C367" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D367" s="10" t="inlineStr">
+      <c r="D367" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -16571,7 +16773,7 @@
       <c r="C370" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D370" s="10" t="inlineStr">
+      <c r="D370" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -16599,7 +16801,7 @@
       <c r="C371" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="D371" s="10" t="inlineStr">
+      <c r="D371" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -16655,7 +16857,7 @@
       <c r="C373" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="D373" s="10" t="inlineStr">
+      <c r="D373" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -16823,7 +17025,7 @@
       <c r="C379" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="D379" s="10" t="inlineStr">
+      <c r="D379" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -17103,7 +17305,7 @@
       <c r="C389" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="D389" s="10" t="inlineStr">
+      <c r="D389" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -17159,7 +17361,7 @@
       <c r="C391" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="D391" s="12" t="inlineStr">
+      <c r="D391" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -17215,7 +17417,7 @@
       <c r="C393" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D393" s="12" t="inlineStr">
+      <c r="D393" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -17355,7 +17557,7 @@
       <c r="C398" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D398" s="12" t="inlineStr">
+      <c r="D398" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -17467,7 +17669,7 @@
       <c r="C402" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="D402" s="12" t="inlineStr">
+      <c r="D402" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -17495,7 +17697,7 @@
       <c r="C403" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D403" s="12" t="inlineStr">
+      <c r="D403" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -17523,7 +17725,7 @@
       <c r="C404" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D404" s="10" t="inlineStr">
+      <c r="D404" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -18083,7 +18285,7 @@
       <c r="C424" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="D424" s="12" t="inlineStr">
+      <c r="D424" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -18167,7 +18369,7 @@
       <c r="C427" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="D427" s="10" t="inlineStr">
+      <c r="D427" s="11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -18195,7 +18397,7 @@
       <c r="C428" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D428" s="12" t="inlineStr">
+      <c r="D428" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -18223,7 +18425,7 @@
       <c r="C429" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="D429" s="12" t="inlineStr">
+      <c r="D429" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -18251,7 +18453,7 @@
       <c r="C430" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D430" s="12" t="inlineStr">
+      <c r="D430" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -18419,7 +18621,7 @@
       <c r="C436" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="D436" s="12" t="inlineStr">
+      <c r="D436" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -18447,7 +18649,7 @@
       <c r="C437" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D437" s="12" t="inlineStr">
+      <c r="D437" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -18783,7 +18985,7 @@
       <c r="C449" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D449" s="12" t="inlineStr">
+      <c r="D449" s="16" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
@@ -21714,16 +21916,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>REMOVED  (10 articles)</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n"/>
-      <c r="C2" s="15" t="n"/>
-      <c r="D2" s="15" t="n"/>
-      <c r="E2" s="15" t="n"/>
-      <c r="F2" s="15" t="n"/>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr"/>
@@ -21986,16 +22188,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>ADDED IN THEIR PLACE  (10 articles)</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="17" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="21" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr"/>
@@ -22258,20 +22460,20 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>KEPT, NEW ANGLE  (3 articles)</t>
         </is>
       </c>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
+      <c r="B24" s="23" t="n"/>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
+      <c r="F24" s="23" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="2" t="inlineStr"/>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="24" t="inlineStr">
         <is>
           <t>was:  The Girlie Vault Guide to Flare Leggings
 now:  Legging Cuts, Compared: Flare, Straight, Capri and Bike Short</t>
@@ -22298,7 +22500,7 @@
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="24" t="inlineStr">
         <is>
           <t>was:  Tankini Swimsuits: How to Find Your Perfect Fit
 now:  One-Piece, Tankini or Bikini: Which Swimsuit Suits You</t>
@@ -22325,7 +22527,7 @@
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>was:  Plus-Size Workout Clothes for Confident Movement
 now:  Plus-Size Activewear That Moves: A Fit and Fabric Guide</t>
@@ -22351,34 +22553,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="25" t="inlineStr">
         <is>
           <t>YOUR EXISTING BLOG PAGES  (nothing goes live without your review)</t>
         </is>
       </c>
-      <c r="B28" s="22" t="n"/>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
-      <c r="F28" s="22" t="n"/>
+      <c r="B28" s="26" t="n"/>
+      <c r="C28" s="26" t="n"/>
+      <c r="D28" s="26" t="n"/>
+      <c r="E28" s="26" t="n"/>
+      <c r="F28" s="26" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>Page</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="C29" s="27" t="inlineStr">
         <is>
           <t>Google, last 90 days</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F29" s="23" t="inlineStr">
+      <c r="F29" s="27" t="inlineStr">
         <is>
           <t>What we propose and why</t>
         </is>
@@ -22402,7 +22604,7 @@
           <t>Going ahead</t>
         </is>
       </c>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="F30" s="24" t="inlineStr">
         <is>
           <t>New title and description in Google only; the article itself stays as is. The page already ranks on page 1, the current headline undersells it.</t>
         </is>
@@ -22426,7 +22628,7 @@
           <t>Going ahead</t>
         </is>
       </c>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="F31" s="24" t="inlineStr">
         <is>
           <t>Full rewrite built around the questions people actually type, like 'how do you wear high waisted leggings'. Sits on page 2 today with zero clicks.</t>
         </is>
@@ -22450,14 +22652,14 @@
           <t>Awaiting your OK</t>
         </is>
       </c>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="F32" s="24" t="inlineStr">
         <is>
           <t>Merge its best content into How to Wear Leggings and redirect the old address there. The two pages currently compete for the same searches, so Google shows neither one well. Every old link keeps working.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="138" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="28" t="inlineStr">
         <is>
           <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
 On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
@@ -22487,30 +22689,30 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Girlie Vault — Keyword Research Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>Companion to your SEO Growth Roadmap. Built from SEMrush Keyword Strategy Builder + Keyword Gap (US).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>What's in this workbook</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
-        <is>
-          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD).
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD). Rows added or re-angled since your July plan are tinted and flagged in the Changed column.
 2. Keyword Universe    · the broader research surfaced from SEMrush; keywords already in the plan are flagged 'Yes (planned)', the rest are 'Overflow' opportunities for later months.
 3. Excluded            · high-volume keywords we intentionally left out, with the reason for each.
 4. Plan Changes        · every article swapped or re-angled since the plan you approved in July, plus the four pages that already exist on your blog and what we have proposed for each.
@@ -22519,14 +22721,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>How to read difficulty (KD)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>KD is SEMrush's 0-100 ranking-difficulty score. We front-load easy wins for a young domain:
   Very Easy (&lt;15) · Easy (15-29) · Moderate (30-44) · Hard (45+).
@@ -22535,14 +22737,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>The six content pillars</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Leggings &amp; Bottoms      · your largest commercial cluster (leggings with pockets, seamless, compression, biker shorts).
 Swimwear &amp; Beach        · one-piece, bikini sets, prints and patterns, rash guards.
@@ -22554,14 +22756,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Funnel philosophy</t>
         </is>
       </c>
     </row>
     <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>BoFu (50) · category buying guides for shoppers ready to purchase.
 MoFu (51) · best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
@@ -22571,14 +22773,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>What we excluded, and why</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>See the 'Excluded' tab for the full list. The big categories:
   Menswear / couples        · off-audience for a women's brand.
@@ -22591,28 +22793,28 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Working titles</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Headlines in the Article Plan are working titles: the keyword, angle and funnel stage are locked, but the exact wording is finalized at production with an SEO title-lock pass. Your input on titles is welcome.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>Approve the plan and ClusterMagic begins the Month 1 batch. Articles are entity-rich, internally linked, schema-marked, and shipped to your store as drafts for review. The Reddit/AEO layer runs alongside to start earning brand mentions in AI answers.</t>
         </is>

</xml_diff>

<commit_message>
girlievault: workbook lists removed July articles in red under the plan
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,16 @@
       <sz val="10"/>
     </font>
     <font>
+      <strike val="1"/>
+      <color rgb="007A4A46"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B3261E"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="10"/>
     </font>
@@ -72,7 +82,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -156,6 +166,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FDECEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001A73E8"/>
       </patternFill>
     </fill>
@@ -186,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -209,6 +224,9 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -216,15 +234,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -590,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6402,6 +6420,513 @@
         </is>
       </c>
       <c r="K121" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="18" t="inlineStr">
+        <is>
+          <t>REMOVED FROM THE JULY PLAN  (why: see the Plan Changes tab)</t>
+        </is>
+      </c>
+      <c r="B123" s="19" t="n"/>
+      <c r="C123" s="19" t="n"/>
+      <c r="D123" s="19" t="n"/>
+      <c r="E123" s="19" t="n"/>
+      <c r="F123" s="19" t="n"/>
+      <c r="G123" s="19" t="n"/>
+      <c r="H123" s="19" t="n"/>
+      <c r="I123" s="19" t="n"/>
+      <c r="J123" s="19" t="n"/>
+      <c r="K123" s="19" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="20" t="inlineStr"/>
+      <c r="B124" s="20" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C124" s="21" t="inlineStr">
+        <is>
+          <t>Workout Sets: The Girlie Vault Guide to Matched Activewear</t>
+        </is>
+      </c>
+      <c r="D124" s="20" t="inlineStr">
+        <is>
+          <t>workout sets</t>
+        </is>
+      </c>
+      <c r="E124" s="20" t="inlineStr">
+        <is>
+          <t>Matching Sets &amp; Outfits</t>
+        </is>
+      </c>
+      <c r="F124" s="20" t="inlineStr">
+        <is>
+          <t>BoFu</t>
+        </is>
+      </c>
+      <c r="G124" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H124" s="20" t="n">
+        <v>40500</v>
+      </c>
+      <c r="I124" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="J124" s="20" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="K124" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="20" t="inlineStr"/>
+      <c r="B125" s="20" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C125" s="21" t="inlineStr">
+        <is>
+          <t>Swim Shorts for Women: Comfort Meets Coverage</t>
+        </is>
+      </c>
+      <c r="D125" s="20" t="inlineStr">
+        <is>
+          <t>swim shorts for women</t>
+        </is>
+      </c>
+      <c r="E125" s="20" t="inlineStr">
+        <is>
+          <t>Swimwear &amp; Beach</t>
+        </is>
+      </c>
+      <c r="F125" s="20" t="inlineStr">
+        <is>
+          <t>MoFu</t>
+        </is>
+      </c>
+      <c r="G125" s="20" t="inlineStr">
+        <is>
+          <t>Transactional</t>
+        </is>
+      </c>
+      <c r="H125" s="20" t="n">
+        <v>12100</v>
+      </c>
+      <c r="I125" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="J125" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="K125" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="20" t="inlineStr"/>
+      <c r="B126" s="20" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C126" s="21" t="inlineStr">
+        <is>
+          <t>Swim Skirts: Flattering Coverage for Beach and Pool</t>
+        </is>
+      </c>
+      <c r="D126" s="20" t="inlineStr">
+        <is>
+          <t>swim skirt</t>
+        </is>
+      </c>
+      <c r="E126" s="20" t="inlineStr">
+        <is>
+          <t>Swimwear &amp; Beach</t>
+        </is>
+      </c>
+      <c r="F126" s="20" t="inlineStr">
+        <is>
+          <t>BoFu</t>
+        </is>
+      </c>
+      <c r="G126" s="20" t="inlineStr">
+        <is>
+          <t>Transactional</t>
+        </is>
+      </c>
+      <c r="H126" s="20" t="n">
+        <v>8100</v>
+      </c>
+      <c r="I126" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="J126" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="K126" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="20" t="inlineStr"/>
+      <c r="B127" s="20" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C127" s="21" t="inlineStr">
+        <is>
+          <t>Tankini Beachwear: Coverage and Confidence in One</t>
+        </is>
+      </c>
+      <c r="D127" s="20" t="inlineStr">
+        <is>
+          <t>tankini beachwear</t>
+        </is>
+      </c>
+      <c r="E127" s="20" t="inlineStr">
+        <is>
+          <t>Swimwear &amp; Beach</t>
+        </is>
+      </c>
+      <c r="F127" s="20" t="inlineStr">
+        <is>
+          <t>BoFu</t>
+        </is>
+      </c>
+      <c r="G127" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H127" s="20" t="n">
+        <v>6600</v>
+      </c>
+      <c r="I127" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="J127" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="K127" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="20" t="inlineStr"/>
+      <c r="B128" s="20" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C128" s="21" t="inlineStr">
+        <is>
+          <t>High-Waisted Leggings for All-Day Comfort and Support</t>
+        </is>
+      </c>
+      <c r="D128" s="20" t="inlineStr">
+        <is>
+          <t>high waisted leggings</t>
+        </is>
+      </c>
+      <c r="E128" s="20" t="inlineStr">
+        <is>
+          <t>Leggings &amp; Bottoms</t>
+        </is>
+      </c>
+      <c r="F128" s="20" t="inlineStr">
+        <is>
+          <t>MoFu</t>
+        </is>
+      </c>
+      <c r="G128" s="20" t="inlineStr">
+        <is>
+          <t>Transactional</t>
+        </is>
+      </c>
+      <c r="H128" s="20" t="n">
+        <v>6600</v>
+      </c>
+      <c r="I128" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="J128" s="20" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="K128" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="20" t="inlineStr"/>
+      <c r="B129" s="20" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C129" s="21" t="inlineStr">
+        <is>
+          <t>Women's Board Shorts: Active Coverage for Sun and Surf</t>
+        </is>
+      </c>
+      <c r="D129" s="20" t="inlineStr">
+        <is>
+          <t>womens board shorts</t>
+        </is>
+      </c>
+      <c r="E129" s="20" t="inlineStr">
+        <is>
+          <t>Leggings &amp; Bottoms</t>
+        </is>
+      </c>
+      <c r="F129" s="20" t="inlineStr">
+        <is>
+          <t>BoFu</t>
+        </is>
+      </c>
+      <c r="G129" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H129" s="20" t="n">
+        <v>5400</v>
+      </c>
+      <c r="I129" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="J129" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="K129" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="20" t="inlineStr"/>
+      <c r="B130" s="20" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="C130" s="21" t="inlineStr">
+        <is>
+          <t>Seamless Leggings for a Smooth, Sculpted Fit</t>
+        </is>
+      </c>
+      <c r="D130" s="20" t="inlineStr">
+        <is>
+          <t>seamless leggings</t>
+        </is>
+      </c>
+      <c r="E130" s="20" t="inlineStr">
+        <is>
+          <t>Leggings &amp; Bottoms</t>
+        </is>
+      </c>
+      <c r="F130" s="20" t="inlineStr">
+        <is>
+          <t>MoFu</t>
+        </is>
+      </c>
+      <c r="G130" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H130" s="20" t="n">
+        <v>4400</v>
+      </c>
+      <c r="I130" s="20" t="n">
+        <v>31</v>
+      </c>
+      <c r="J130" s="20" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="K130" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="20" t="inlineStr"/>
+      <c r="B131" s="20" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C131" s="21" t="inlineStr">
+        <is>
+          <t>Women's Tracksuit Pants: How to Choose Your Fit</t>
+        </is>
+      </c>
+      <c r="D131" s="20" t="inlineStr">
+        <is>
+          <t>tracksuit pants for ladies</t>
+        </is>
+      </c>
+      <c r="E131" s="20" t="inlineStr">
+        <is>
+          <t>Leggings &amp; Bottoms</t>
+        </is>
+      </c>
+      <c r="F131" s="20" t="inlineStr">
+        <is>
+          <t>BoFu</t>
+        </is>
+      </c>
+      <c r="G131" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H131" s="20" t="n">
+        <v>3600</v>
+      </c>
+      <c r="I131" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="J131" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="K131" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="20" t="inlineStr"/>
+      <c r="B132" s="20" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C132" s="21" t="inlineStr">
+        <is>
+          <t>How to Style Yoga Flare Pants for Any Occasion</t>
+        </is>
+      </c>
+      <c r="D132" s="20" t="inlineStr">
+        <is>
+          <t>yoga flare pants outfits</t>
+        </is>
+      </c>
+      <c r="E132" s="20" t="inlineStr">
+        <is>
+          <t>Matching Sets &amp; Outfits</t>
+        </is>
+      </c>
+      <c r="F132" s="20" t="inlineStr">
+        <is>
+          <t>ToFu</t>
+        </is>
+      </c>
+      <c r="G132" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H132" s="20" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I132" s="20" t="n">
+        <v>24</v>
+      </c>
+      <c r="J132" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="K132" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="20" t="inlineStr"/>
+      <c r="B133" s="20" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C133" s="21" t="inlineStr">
+        <is>
+          <t>The Best Seamless Sports Bras for Everyday Comfort</t>
+        </is>
+      </c>
+      <c r="D133" s="20" t="inlineStr">
+        <is>
+          <t>seamless sports bra</t>
+        </is>
+      </c>
+      <c r="E133" s="20" t="inlineStr">
+        <is>
+          <t>Sports Bras &amp; Tops</t>
+        </is>
+      </c>
+      <c r="F133" s="20" t="inlineStr">
+        <is>
+          <t>MoFu</t>
+        </is>
+      </c>
+      <c r="G133" s="20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H133" s="20" t="n">
+        <v>1300</v>
+      </c>
+      <c r="I133" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="J133" s="20" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="K133" s="22" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22188,16 +22713,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>ADDED IN THEIR PLACE  (10 articles)</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="21" t="n"/>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="24" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr"/>
@@ -22460,20 +22985,20 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>KEPT, NEW ANGLE  (3 articles)</t>
         </is>
       </c>
-      <c r="B24" s="23" t="n"/>
-      <c r="C24" s="23" t="n"/>
-      <c r="D24" s="23" t="n"/>
-      <c r="E24" s="23" t="n"/>
-      <c r="F24" s="23" t="n"/>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="26" t="n"/>
+      <c r="D24" s="26" t="n"/>
+      <c r="E24" s="26" t="n"/>
+      <c r="F24" s="26" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="2" t="inlineStr"/>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>was:  The Girlie Vault Guide to Flare Leggings
 now:  Legging Cuts, Compared: Flare, Straight, Capri and Bike Short</t>
@@ -22500,7 +23025,7 @@
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>was:  Tankini Swimsuits: How to Find Your Perfect Fit
 now:  One-Piece, Tankini or Bikini: Which Swimsuit Suits You</t>
@@ -22527,7 +23052,7 @@
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>was:  Plus-Size Workout Clothes for Confident Movement
 now:  Plus-Size Activewear That Moves: A Fit and Fabric Guide</t>
@@ -22553,34 +23078,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="inlineStr">
+      <c r="A28" s="28" t="inlineStr">
         <is>
           <t>YOUR EXISTING BLOG PAGES  (nothing goes live without your review)</t>
         </is>
       </c>
-      <c r="B28" s="26" t="n"/>
-      <c r="C28" s="26" t="n"/>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="26" t="n"/>
-      <c r="F28" s="26" t="n"/>
+      <c r="B28" s="29" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="29" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B29" s="30" t="inlineStr">
         <is>
           <t>Page</t>
         </is>
       </c>
-      <c r="C29" s="27" t="inlineStr">
+      <c r="C29" s="30" t="inlineStr">
         <is>
           <t>Google, last 90 days</t>
         </is>
       </c>
-      <c r="E29" s="27" t="inlineStr">
+      <c r="E29" s="30" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F29" s="27" t="inlineStr">
+      <c r="F29" s="30" t="inlineStr">
         <is>
           <t>What we propose and why</t>
         </is>
@@ -22604,7 +23129,7 @@
           <t>Going ahead</t>
         </is>
       </c>
-      <c r="F30" s="24" t="inlineStr">
+      <c r="F30" s="27" t="inlineStr">
         <is>
           <t>New title and description in Google only; the article itself stays as is. The page already ranks on page 1, the current headline undersells it.</t>
         </is>
@@ -22628,7 +23153,7 @@
           <t>Going ahead</t>
         </is>
       </c>
-      <c r="F31" s="24" t="inlineStr">
+      <c r="F31" s="27" t="inlineStr">
         <is>
           <t>Full rewrite built around the questions people actually type, like 'how do you wear high waisted leggings'. Sits on page 2 today with zero clicks.</t>
         </is>
@@ -22652,14 +23177,14 @@
           <t>Awaiting your OK</t>
         </is>
       </c>
-      <c r="F32" s="24" t="inlineStr">
+      <c r="F32" s="27" t="inlineStr">
         <is>
           <t>Merge its best content into How to Wear Leggings and redirect the old address there. The two pages currently compete for the same searches, so Google shows neither one well. Every old link keeps working.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="138" customHeight="1">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="31" t="inlineStr">
         <is>
           <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
 On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
@@ -22689,30 +23214,30 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>Girlie Vault — Keyword Research Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>Companion to your SEO Growth Roadmap. Built from SEMrush Keyword Strategy Builder + Keyword Gap (US).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>What's in this workbook</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD). Rows added or re-angled since your July plan are tinted and flagged in the Changed column.
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD). Rows added or re-angled since your July plan are tinted and flagged in the Changed column, and the articles removed from the July plan sit under the 120 in red.
 2. Keyword Universe    · the broader research surfaced from SEMrush; keywords already in the plan are flagged 'Yes (planned)', the rest are 'Overflow' opportunities for later months.
 3. Excluded            · high-volume keywords we intentionally left out, with the reason for each.
 4. Plan Changes        · every article swapped or re-angled since the plan you approved in July, plus the four pages that already exist on your blog and what we have proposed for each.
@@ -22721,14 +23246,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="34" t="inlineStr">
         <is>
           <t>How to read difficulty (KD)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>KD is SEMrush's 0-100 ranking-difficulty score. We front-load easy wins for a young domain:
   Very Easy (&lt;15) · Easy (15-29) · Moderate (30-44) · Hard (45+).
@@ -22737,14 +23262,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>The six content pillars</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Leggings &amp; Bottoms      · your largest commercial cluster (leggings with pockets, seamless, compression, biker shorts).
 Swimwear &amp; Beach        · one-piece, bikini sets, prints and patterns, rash guards.
@@ -22756,14 +23281,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="34" t="inlineStr">
         <is>
           <t>Funnel philosophy</t>
         </is>
       </c>
     </row>
     <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>BoFu (50) · category buying guides for shoppers ready to purchase.
 MoFu (51) · best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
@@ -22773,14 +23298,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="34" t="inlineStr">
         <is>
           <t>What we excluded, and why</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>See the 'Excluded' tab for the full list. The big categories:
   Menswear / couples        · off-audience for a women's brand.
@@ -22793,28 +23318,28 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t>Working titles</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Headlines in the Article Plan are working titles: the keyword, angle and funnel stage are locked, but the exact wording is finalized at production with an SEO title-lock pass. Your input on titles is welcome.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Approve the plan and ClusterMagic begins the Month 1 batch. Articles are entity-rich, internally linked, schema-marked, and shipped to your store as drafts for review. The Reddit/AEO layer runs alongside to start earning brand mentions in AI answers.</t>
         </is>

</xml_diff>

<commit_message>
girlievault: workbook shows page updates at the bottom of Article Plan
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001A73E8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -82,7 +87,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -174,6 +179,11 @@
         <fgColor rgb="001A73E8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -201,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -227,6 +237,10 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,15 +248,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -608,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K133"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6925,6 +6937,98 @@
       <c r="K133" s="22" t="inlineStr">
         <is>
           <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="23" t="inlineStr">
+        <is>
+          <t>UPDATES TO YOUR CURRENT PAGES  (details in the Plan Changes tab)</t>
+        </is>
+      </c>
+      <c r="B135" s="24" t="n"/>
+      <c r="C135" s="24" t="n"/>
+      <c r="D135" s="24" t="n"/>
+      <c r="E135" s="24" t="n"/>
+      <c r="F135" s="24" t="n"/>
+      <c r="G135" s="24" t="n"/>
+      <c r="H135" s="24" t="n"/>
+      <c r="I135" s="24" t="n"/>
+      <c r="J135" s="24" t="n"/>
+      <c r="K135" s="24" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="25" t="inlineStr"/>
+      <c r="B136" s="25" t="inlineStr"/>
+      <c r="C136" s="25" t="inlineStr">
+        <is>
+          <t>Finding the Best Leggings for Thick Thighs: A Guide to ...</t>
+        </is>
+      </c>
+      <c r="D136" s="25" t="inlineStr">
+        <is>
+          <t>New title + description</t>
+        </is>
+      </c>
+      <c r="E136" s="25" t="inlineStr"/>
+      <c r="F136" s="25" t="inlineStr"/>
+      <c r="G136" s="25" t="inlineStr"/>
+      <c r="H136" s="25" t="inlineStr"/>
+      <c r="I136" s="25" t="inlineStr"/>
+      <c r="J136" s="25" t="inlineStr"/>
+      <c r="K136" s="26" t="inlineStr">
+        <is>
+          <t>Going ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="25" t="inlineStr"/>
+      <c r="B137" s="25" t="inlineStr"/>
+      <c r="C137" s="25" t="inlineStr">
+        <is>
+          <t>How to Wear Leggings for Any Occasion and Feel Absolutely Confident</t>
+        </is>
+      </c>
+      <c r="D137" s="25" t="inlineStr">
+        <is>
+          <t>Full rewrite</t>
+        </is>
+      </c>
+      <c r="E137" s="25" t="inlineStr"/>
+      <c r="F137" s="25" t="inlineStr"/>
+      <c r="G137" s="25" t="inlineStr"/>
+      <c r="H137" s="25" t="inlineStr"/>
+      <c r="I137" s="25" t="inlineStr"/>
+      <c r="J137" s="25" t="inlineStr"/>
+      <c r="K137" s="26" t="inlineStr">
+        <is>
+          <t>Going ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="25" t="inlineStr"/>
+      <c r="B138" s="25" t="inlineStr"/>
+      <c r="C138" s="25" t="inlineStr">
+        <is>
+          <t>Finding the Best High Waisted Leggings for You</t>
+        </is>
+      </c>
+      <c r="D138" s="25" t="inlineStr">
+        <is>
+          <t>Merge into How to Wear Leggings</t>
+        </is>
+      </c>
+      <c r="E138" s="25" t="inlineStr"/>
+      <c r="F138" s="25" t="inlineStr"/>
+      <c r="G138" s="25" t="inlineStr"/>
+      <c r="H138" s="25" t="inlineStr"/>
+      <c r="I138" s="25" t="inlineStr"/>
+      <c r="J138" s="25" t="inlineStr"/>
+      <c r="K138" s="26" t="inlineStr">
+        <is>
+          <t>Awaiting your OK</t>
         </is>
       </c>
     </row>
@@ -22713,16 +22817,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>ADDED IN THEIR PLACE  (10 articles)</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n"/>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="24" t="n"/>
-      <c r="F13" s="24" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="28" t="n"/>
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="28" t="n"/>
+      <c r="F13" s="28" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr"/>
@@ -22985,20 +23089,20 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>KEPT, NEW ANGLE  (3 articles)</t>
         </is>
       </c>
-      <c r="B24" s="26" t="n"/>
-      <c r="C24" s="26" t="n"/>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="n"/>
-      <c r="F24" s="26" t="n"/>
+      <c r="B24" s="30" t="n"/>
+      <c r="C24" s="30" t="n"/>
+      <c r="D24" s="30" t="n"/>
+      <c r="E24" s="30" t="n"/>
+      <c r="F24" s="30" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="2" t="inlineStr"/>
-      <c r="B25" s="27" t="inlineStr">
+      <c r="B25" s="31" t="inlineStr">
         <is>
           <t>was:  The Girlie Vault Guide to Flare Leggings
 now:  Legging Cuts, Compared: Flare, Straight, Capri and Bike Short</t>
@@ -23025,7 +23129,7 @@
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="27" t="inlineStr">
+      <c r="B26" s="31" t="inlineStr">
         <is>
           <t>was:  Tankini Swimsuits: How to Find Your Perfect Fit
 now:  One-Piece, Tankini or Bikini: Which Swimsuit Suits You</t>
@@ -23052,7 +23156,7 @@
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="27" t="inlineStr">
+      <c r="B27" s="31" t="inlineStr">
         <is>
           <t>was:  Plus-Size Workout Clothes for Confident Movement
 now:  Plus-Size Activewear That Moves: A Fit and Fabric Guide</t>
@@ -23078,34 +23182,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>YOUR EXISTING BLOG PAGES  (nothing goes live without your review)</t>
         </is>
       </c>
-      <c r="B28" s="29" t="n"/>
-      <c r="C28" s="29" t="n"/>
-      <c r="D28" s="29" t="n"/>
-      <c r="E28" s="29" t="n"/>
-      <c r="F28" s="29" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="30" t="inlineStr">
+      <c r="B29" s="32" t="inlineStr">
         <is>
           <t>Page</t>
         </is>
       </c>
-      <c r="C29" s="30" t="inlineStr">
+      <c r="C29" s="32" t="inlineStr">
         <is>
           <t>Google, last 90 days</t>
         </is>
       </c>
-      <c r="E29" s="30" t="inlineStr">
+      <c r="E29" s="32" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F29" s="30" t="inlineStr">
+      <c r="F29" s="32" t="inlineStr">
         <is>
           <t>What we propose and why</t>
         </is>
@@ -23129,7 +23233,7 @@
           <t>Going ahead</t>
         </is>
       </c>
-      <c r="F30" s="27" t="inlineStr">
+      <c r="F30" s="31" t="inlineStr">
         <is>
           <t>New title and description in Google only; the article itself stays as is. The page already ranks on page 1, the current headline undersells it.</t>
         </is>
@@ -23153,7 +23257,7 @@
           <t>Going ahead</t>
         </is>
       </c>
-      <c r="F31" s="27" t="inlineStr">
+      <c r="F31" s="31" t="inlineStr">
         <is>
           <t>Full rewrite built around the questions people actually type, like 'how do you wear high waisted leggings'. Sits on page 2 today with zero clicks.</t>
         </is>
@@ -23177,14 +23281,14 @@
           <t>Awaiting your OK</t>
         </is>
       </c>
-      <c r="F32" s="27" t="inlineStr">
+      <c r="F32" s="31" t="inlineStr">
         <is>
           <t>Merge its best content into How to Wear Leggings and redirect the old address there. The two pages currently compete for the same searches, so Google shows neither one well. Every old link keeps working.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="138" customHeight="1">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="A34" s="33" t="inlineStr">
         <is>
           <t>10 articles replaced and 3 re-angled, out of 120. Everything else is unchanged from the plan you approved, and the count per month is still 40 / 40 / 40.
 On the numbers: the removed articles carried 91,000 monthly searches and the new ones carry 36,300, which looks like a step down until you split it. 47,100 of it sits on two terms your site already ranks for, so that traffic was never ours to win twice. The other 43,900 was demand for products you do not sell, where ranking sends a shopper to a page that cannot serve her. The 36,300 coming in is demand for things in your catalogue.
@@ -23214,30 +23318,30 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>Girlie Vault — Keyword Research Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>Companion to your SEO Growth Roadmap. Built from SEMrush Keyword Strategy Builder + Keyword Gap (US).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="34" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>What's in this workbook</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
-        <is>
-          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD). Rows added or re-angled since your July plan are tinted and flagged in the Changed column, and the articles removed from the July plan sit under the 120 in red.
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>1. Article Plan        · the 120 articles selected for the 3-month plan, mapped to month, pillar, funnel stage, volume and difficulty (KD). Rows added or re-angled since your July plan are tinted and flagged in the Changed column, and the articles removed from the July plan sit under the 120 in red, with the three proposed updates to your existing pages at the very bottom.
 2. Keyword Universe    · the broader research surfaced from SEMrush; keywords already in the plan are flagged 'Yes (planned)', the rest are 'Overflow' opportunities for later months.
 3. Excluded            · high-volume keywords we intentionally left out, with the reason for each.
 4. Plan Changes        · every article swapped or re-angled since the plan you approved in July, plus the four pages that already exist on your blog and what we have proposed for each.
@@ -23246,14 +23350,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>How to read difficulty (KD)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>KD is SEMrush's 0-100 ranking-difficulty score. We front-load easy wins for a young domain:
   Very Easy (&lt;15) · Easy (15-29) · Moderate (30-44) · Hard (45+).
@@ -23262,14 +23366,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="34" t="inlineStr">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>The six content pillars</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>Leggings &amp; Bottoms      · your largest commercial cluster (leggings with pockets, seamless, compression, biker shorts).
 Swimwear &amp; Beach        · one-piece, bikini sets, prints and patterns, rash guards.
@@ -23281,14 +23385,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="34" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>Funnel philosophy</t>
         </is>
       </c>
     </row>
     <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>BoFu (50) · category buying guides for shoppers ready to purchase.
 MoFu (51) · best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
@@ -23298,14 +23402,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="34" t="inlineStr">
+      <c r="A16" s="36" t="inlineStr">
         <is>
           <t>What we excluded, and why</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="33" t="inlineStr">
         <is>
           <t>See the 'Excluded' tab for the full list. The big categories:
   Menswear / couples        · off-audience for a women's brand.
@@ -23318,28 +23422,28 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="36" t="inlineStr">
         <is>
           <t>Working titles</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>Headlines in the Article Plan are working titles: the keyword, angle and funnel stage are locked, but the exact wording is finalized at production with an SEO title-lock pass. Your input on titles is welcome.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="34" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
         <is>
           <t>Approve the plan and ClusterMagic begins the Month 1 batch. Articles are entity-rich, internally linked, schema-marked, and shipped to your store as drafts for review. The Reddit/AEO layer runs alongside to start earning brand mentions in AI answers.</t>
         </is>

</xml_diff>